<commit_message>
Add Appium and Vulnerability testing workflows, update backend submodule reference, and commit updated reports
</commit_message>
<xml_diff>
--- a/sentinel-android/testing/excel-reports/Sentinel_Appium_Test_Report.xlsx
+++ b/sentinel-android/testing/excel-reports/Sentinel_Appium_Test_Report.xlsx
@@ -645,7 +645,7 @@
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>51.58s</t>
+          <t>49.17s</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="H7" s="11" t="inlineStr">
         <is>
-          <t>9.94s</t>
+          <t>10.88s</t>
         </is>
       </c>
     </row>
@@ -703,7 +703,7 @@
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>11.42s</t>
+          <t>8.47s</t>
         </is>
       </c>
     </row>
@@ -732,7 +732,7 @@
       </c>
       <c r="H9" s="11" t="inlineStr">
         <is>
-          <t>13.54s</t>
+          <t>15.37s</t>
         </is>
       </c>
     </row>
@@ -761,7 +761,7 @@
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>13.85s</t>
+          <t>12.03s</t>
         </is>
       </c>
     </row>
@@ -790,7 +790,7 @@
       </c>
       <c r="H11" s="11" t="inlineStr">
         <is>
-          <t>14.55s</t>
+          <t>15.95s</t>
         </is>
       </c>
     </row>
@@ -819,7 +819,7 @@
       </c>
       <c r="H12" s="14" t="inlineStr">
         <is>
-          <t>114.88s</t>
+          <t>111.87s</t>
         </is>
       </c>
     </row>
@@ -1102,7 +1102,7 @@
       </c>
       <c r="K2" s="7" t="inlineStr">
         <is>
-          <t>1.24s</t>
+          <t>0.28s</t>
         </is>
       </c>
       <c r="L2" s="15" t="inlineStr">
@@ -1172,7 +1172,7 @@
       </c>
       <c r="K3" s="11" t="inlineStr">
         <is>
-          <t>1.20s</t>
+          <t>0.64s</t>
         </is>
       </c>
       <c r="L3" s="17" t="inlineStr">
@@ -1242,7 +1242,7 @@
       </c>
       <c r="K4" s="7" t="inlineStr">
         <is>
-          <t>1.23s</t>
+          <t>0.76s</t>
         </is>
       </c>
       <c r="L4" s="15" t="inlineStr">
@@ -1312,7 +1312,7 @@
       </c>
       <c r="K5" s="11" t="inlineStr">
         <is>
-          <t>0.89s</t>
+          <t>0.57s</t>
         </is>
       </c>
       <c r="L5" s="17" t="inlineStr">
@@ -1382,7 +1382,7 @@
       </c>
       <c r="K6" s="7" t="inlineStr">
         <is>
-          <t>0.86s</t>
+          <t>0.33s</t>
         </is>
       </c>
       <c r="L6" s="15" t="inlineStr">
@@ -1452,7 +1452,7 @@
       </c>
       <c r="K7" s="11" t="inlineStr">
         <is>
-          <t>0.64s</t>
+          <t>0.13s</t>
         </is>
       </c>
       <c r="L7" s="17" t="inlineStr">
@@ -1522,7 +1522,7 @@
       </c>
       <c r="K8" s="7" t="inlineStr">
         <is>
-          <t>0.52s</t>
+          <t>0.98s</t>
         </is>
       </c>
       <c r="L8" s="15" t="inlineStr">
@@ -1592,7 +1592,7 @@
       </c>
       <c r="K9" s="11" t="inlineStr">
         <is>
-          <t>0.95s</t>
+          <t>0.43s</t>
         </is>
       </c>
       <c r="L9" s="17" t="inlineStr">
@@ -1662,7 +1662,7 @@
       </c>
       <c r="K10" s="7" t="inlineStr">
         <is>
-          <t>0.16s</t>
+          <t>1.03s</t>
         </is>
       </c>
       <c r="L10" s="15" t="inlineStr">
@@ -1732,7 +1732,7 @@
       </c>
       <c r="K11" s="11" t="inlineStr">
         <is>
-          <t>1.03s</t>
+          <t>0.99s</t>
         </is>
       </c>
       <c r="L11" s="17" t="inlineStr">
@@ -1802,7 +1802,7 @@
       </c>
       <c r="K12" s="7" t="inlineStr">
         <is>
-          <t>0.48s</t>
+          <t>0.42s</t>
         </is>
       </c>
       <c r="L12" s="15" t="inlineStr">
@@ -1872,7 +1872,7 @@
       </c>
       <c r="K13" s="11" t="inlineStr">
         <is>
-          <t>0.80s</t>
+          <t>1.19s</t>
         </is>
       </c>
       <c r="L13" s="17" t="inlineStr">
@@ -1942,7 +1942,7 @@
       </c>
       <c r="K14" s="7" t="inlineStr">
         <is>
-          <t>0.26s</t>
+          <t>0.45s</t>
         </is>
       </c>
       <c r="L14" s="15" t="inlineStr">
@@ -2012,7 +2012,7 @@
       </c>
       <c r="K15" s="11" t="inlineStr">
         <is>
-          <t>0.71s</t>
+          <t>1.16s</t>
         </is>
       </c>
       <c r="L15" s="17" t="inlineStr">
@@ -2082,7 +2082,7 @@
       </c>
       <c r="K16" s="7" t="inlineStr">
         <is>
-          <t>0.98s</t>
+          <t>1.02s</t>
         </is>
       </c>
       <c r="L16" s="15" t="inlineStr">
@@ -2152,7 +2152,7 @@
       </c>
       <c r="K17" s="11" t="inlineStr">
         <is>
-          <t>1.07s</t>
+          <t>1.20s</t>
         </is>
       </c>
       <c r="L17" s="17" t="inlineStr">
@@ -2222,7 +2222,7 @@
       </c>
       <c r="K18" s="7" t="inlineStr">
         <is>
-          <t>1.03s</t>
+          <t>0.71s</t>
         </is>
       </c>
       <c r="L18" s="15" t="inlineStr">
@@ -2292,7 +2292,7 @@
       </c>
       <c r="K19" s="11" t="inlineStr">
         <is>
-          <t>1.08s</t>
+          <t>0.43s</t>
         </is>
       </c>
       <c r="L19" s="17" t="inlineStr">
@@ -2362,7 +2362,7 @@
       </c>
       <c r="K20" s="7" t="inlineStr">
         <is>
-          <t>0.59s</t>
+          <t>0.47s</t>
         </is>
       </c>
       <c r="L20" s="15" t="inlineStr">
@@ -2432,7 +2432,7 @@
       </c>
       <c r="K21" s="11" t="inlineStr">
         <is>
-          <t>0.60s</t>
+          <t>0.80s</t>
         </is>
       </c>
       <c r="L21" s="17" t="inlineStr">
@@ -2502,7 +2502,7 @@
       </c>
       <c r="K22" s="7" t="inlineStr">
         <is>
-          <t>0.81s</t>
+          <t>1.17s</t>
         </is>
       </c>
       <c r="L22" s="15" t="inlineStr">
@@ -2572,7 +2572,7 @@
       </c>
       <c r="K23" s="11" t="inlineStr">
         <is>
-          <t>0.54s</t>
+          <t>0.90s</t>
         </is>
       </c>
       <c r="L23" s="17" t="inlineStr">
@@ -2642,7 +2642,7 @@
       </c>
       <c r="K24" s="7" t="inlineStr">
         <is>
-          <t>0.92s</t>
+          <t>1.17s</t>
         </is>
       </c>
       <c r="L24" s="15" t="inlineStr">
@@ -2712,7 +2712,7 @@
       </c>
       <c r="K25" s="11" t="inlineStr">
         <is>
-          <t>0.13s</t>
+          <t>0.53s</t>
         </is>
       </c>
       <c r="L25" s="17" t="inlineStr">
@@ -2782,7 +2782,7 @@
       </c>
       <c r="K26" s="7" t="inlineStr">
         <is>
-          <t>0.62s</t>
+          <t>0.63s</t>
         </is>
       </c>
       <c r="L26" s="15" t="inlineStr">
@@ -2852,7 +2852,7 @@
       </c>
       <c r="K27" s="11" t="inlineStr">
         <is>
-          <t>0.86s</t>
+          <t>0.75s</t>
         </is>
       </c>
       <c r="L27" s="17" t="inlineStr">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="K28" s="7" t="inlineStr">
         <is>
-          <t>1.23s</t>
+          <t>0.46s</t>
         </is>
       </c>
       <c r="L28" s="15" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="K29" s="11" t="inlineStr">
         <is>
-          <t>0.98s</t>
+          <t>0.55s</t>
         </is>
       </c>
       <c r="L29" s="17" t="inlineStr">
@@ -3062,7 +3062,7 @@
       </c>
       <c r="K30" s="7" t="inlineStr">
         <is>
-          <t>0.98s</t>
+          <t>0.26s</t>
         </is>
       </c>
       <c r="L30" s="15" t="inlineStr">
@@ -3132,7 +3132,7 @@
       </c>
       <c r="K31" s="11" t="inlineStr">
         <is>
-          <t>0.70s</t>
+          <t>0.62s</t>
         </is>
       </c>
       <c r="L31" s="17" t="inlineStr">
@@ -3202,7 +3202,7 @@
       </c>
       <c r="K32" s="7" t="inlineStr">
         <is>
-          <t>0.30s</t>
+          <t>1.13s</t>
         </is>
       </c>
       <c r="L32" s="15" t="inlineStr">
@@ -3272,7 +3272,7 @@
       </c>
       <c r="K33" s="11" t="inlineStr">
         <is>
-          <t>1.13s</t>
+          <t>0.59s</t>
         </is>
       </c>
       <c r="L33" s="17" t="inlineStr">
@@ -3342,7 +3342,7 @@
       </c>
       <c r="K34" s="7" t="inlineStr">
         <is>
-          <t>1.09s</t>
+          <t>1.05s</t>
         </is>
       </c>
       <c r="L34" s="15" t="inlineStr">
@@ -3412,7 +3412,7 @@
       </c>
       <c r="K35" s="11" t="inlineStr">
         <is>
-          <t>1.08s</t>
+          <t>0.35s</t>
         </is>
       </c>
       <c r="L35" s="17" t="inlineStr">
@@ -3482,7 +3482,7 @@
       </c>
       <c r="K36" s="7" t="inlineStr">
         <is>
-          <t>0.50s</t>
+          <t>0.17s</t>
         </is>
       </c>
       <c r="L36" s="15" t="inlineStr">
@@ -3552,7 +3552,7 @@
       </c>
       <c r="K37" s="11" t="inlineStr">
         <is>
-          <t>0.42s</t>
+          <t>0.15s</t>
         </is>
       </c>
       <c r="L37" s="17" t="inlineStr">
@@ -3622,7 +3622,7 @@
       </c>
       <c r="K38" s="7" t="inlineStr">
         <is>
-          <t>0.43s</t>
+          <t>0.90s</t>
         </is>
       </c>
       <c r="L38" s="15" t="inlineStr">
@@ -3692,7 +3692,7 @@
       </c>
       <c r="K39" s="11" t="inlineStr">
         <is>
-          <t>0.50s</t>
+          <t>1.00s</t>
         </is>
       </c>
       <c r="L39" s="17" t="inlineStr">
@@ -3762,7 +3762,7 @@
       </c>
       <c r="K40" s="7" t="inlineStr">
         <is>
-          <t>0.21s</t>
+          <t>1.21s</t>
         </is>
       </c>
       <c r="L40" s="15" t="inlineStr">
@@ -3832,7 +3832,7 @@
       </c>
       <c r="K41" s="11" t="inlineStr">
         <is>
-          <t>0.74s</t>
+          <t>0.85s</t>
         </is>
       </c>
       <c r="L41" s="17" t="inlineStr">
@@ -3902,7 +3902,7 @@
       </c>
       <c r="K42" s="7" t="inlineStr">
         <is>
-          <t>0.92s</t>
+          <t>0.20s</t>
         </is>
       </c>
       <c r="L42" s="15" t="inlineStr">
@@ -3972,7 +3972,7 @@
       </c>
       <c r="K43" s="11" t="inlineStr">
         <is>
-          <t>0.35s</t>
+          <t>1.16s</t>
         </is>
       </c>
       <c r="L43" s="17" t="inlineStr">
@@ -4042,7 +4042,7 @@
       </c>
       <c r="K44" s="7" t="inlineStr">
         <is>
-          <t>0.27s</t>
+          <t>0.14s</t>
         </is>
       </c>
       <c r="L44" s="15" t="inlineStr">
@@ -4112,7 +4112,7 @@
       </c>
       <c r="K45" s="11" t="inlineStr">
         <is>
-          <t>0.65s</t>
+          <t>0.29s</t>
         </is>
       </c>
       <c r="L45" s="17" t="inlineStr">
@@ -4182,7 +4182,7 @@
       </c>
       <c r="K46" s="7" t="inlineStr">
         <is>
-          <t>0.90s</t>
+          <t>0.81s</t>
         </is>
       </c>
       <c r="L46" s="15" t="inlineStr">
@@ -4252,7 +4252,7 @@
       </c>
       <c r="K47" s="11" t="inlineStr">
         <is>
-          <t>0.42s</t>
+          <t>0.66s</t>
         </is>
       </c>
       <c r="L47" s="17" t="inlineStr">
@@ -4322,7 +4322,7 @@
       </c>
       <c r="K48" s="7" t="inlineStr">
         <is>
-          <t>0.74s</t>
+          <t>0.87s</t>
         </is>
       </c>
       <c r="L48" s="15" t="inlineStr">
@@ -4392,7 +4392,7 @@
       </c>
       <c r="K49" s="11" t="inlineStr">
         <is>
-          <t>1.22s</t>
+          <t>0.82s</t>
         </is>
       </c>
       <c r="L49" s="17" t="inlineStr">
@@ -4462,7 +4462,7 @@
       </c>
       <c r="K50" s="7" t="inlineStr">
         <is>
-          <t>0.61s</t>
+          <t>0.34s</t>
         </is>
       </c>
       <c r="L50" s="15" t="inlineStr">
@@ -4532,7 +4532,7 @@
       </c>
       <c r="K51" s="11" t="inlineStr">
         <is>
-          <t>0.13s</t>
+          <t>0.83s</t>
         </is>
       </c>
       <c r="L51" s="17" t="inlineStr">
@@ -4602,7 +4602,7 @@
       </c>
       <c r="K52" s="7" t="inlineStr">
         <is>
-          <t>0.36s</t>
+          <t>0.69s</t>
         </is>
       </c>
       <c r="L52" s="15" t="inlineStr">
@@ -4672,7 +4672,7 @@
       </c>
       <c r="K53" s="11" t="inlineStr">
         <is>
-          <t>0.51s</t>
+          <t>0.62s</t>
         </is>
       </c>
       <c r="L53" s="17" t="inlineStr">
@@ -4742,7 +4742,7 @@
       </c>
       <c r="K54" s="7" t="inlineStr">
         <is>
-          <t>1.04s</t>
+          <t>0.70s</t>
         </is>
       </c>
       <c r="L54" s="15" t="inlineStr">
@@ -4812,7 +4812,7 @@
       </c>
       <c r="K55" s="11" t="inlineStr">
         <is>
-          <t>0.90s</t>
+          <t>0.89s</t>
         </is>
       </c>
       <c r="L55" s="17" t="inlineStr">
@@ -4882,7 +4882,7 @@
       </c>
       <c r="K56" s="7" t="inlineStr">
         <is>
-          <t>1.04s</t>
+          <t>0.67s</t>
         </is>
       </c>
       <c r="L56" s="15" t="inlineStr">
@@ -4952,7 +4952,7 @@
       </c>
       <c r="K57" s="11" t="inlineStr">
         <is>
-          <t>0.30s</t>
+          <t>0.19s</t>
         </is>
       </c>
       <c r="L57" s="17" t="inlineStr">
@@ -5022,7 +5022,7 @@
       </c>
       <c r="K58" s="7" t="inlineStr">
         <is>
-          <t>0.64s</t>
+          <t>0.45s</t>
         </is>
       </c>
       <c r="L58" s="15" t="inlineStr">
@@ -5092,7 +5092,7 @@
       </c>
       <c r="K59" s="11" t="inlineStr">
         <is>
-          <t>1.20s</t>
+          <t>0.23s</t>
         </is>
       </c>
       <c r="L59" s="17" t="inlineStr">
@@ -5162,7 +5162,7 @@
       </c>
       <c r="K60" s="7" t="inlineStr">
         <is>
-          <t>1.01s</t>
+          <t>0.55s</t>
         </is>
       </c>
       <c r="L60" s="15" t="inlineStr">
@@ -5232,7 +5232,7 @@
       </c>
       <c r="K61" s="11" t="inlineStr">
         <is>
-          <t>0.73s</t>
+          <t>1.08s</t>
         </is>
       </c>
       <c r="L61" s="17" t="inlineStr">
@@ -5302,7 +5302,7 @@
       </c>
       <c r="K62" s="7" t="inlineStr">
         <is>
-          <t>0.85s</t>
+          <t>1.02s</t>
         </is>
       </c>
       <c r="L62" s="15" t="inlineStr">
@@ -5372,7 +5372,7 @@
       </c>
       <c r="K63" s="11" t="inlineStr">
         <is>
-          <t>0.16s</t>
+          <t>0.42s</t>
         </is>
       </c>
       <c r="L63" s="17" t="inlineStr">
@@ -5442,7 +5442,7 @@
       </c>
       <c r="K64" s="7" t="inlineStr">
         <is>
-          <t>1.02s</t>
+          <t>0.82s</t>
         </is>
       </c>
       <c r="L64" s="15" t="inlineStr">
@@ -5512,7 +5512,7 @@
       </c>
       <c r="K65" s="11" t="inlineStr">
         <is>
-          <t>0.37s</t>
+          <t>0.35s</t>
         </is>
       </c>
       <c r="L65" s="17" t="inlineStr">
@@ -5582,7 +5582,7 @@
       </c>
       <c r="K66" s="7" t="inlineStr">
         <is>
-          <t>0.54s</t>
+          <t>0.14s</t>
         </is>
       </c>
       <c r="L66" s="15" t="inlineStr">
@@ -5652,7 +5652,7 @@
       </c>
       <c r="K67" s="11" t="inlineStr">
         <is>
-          <t>0.32s</t>
+          <t>0.50s</t>
         </is>
       </c>
       <c r="L67" s="17" t="inlineStr">
@@ -5722,7 +5722,7 @@
       </c>
       <c r="K68" s="7" t="inlineStr">
         <is>
-          <t>0.68s</t>
+          <t>1.02s</t>
         </is>
       </c>
       <c r="L68" s="15" t="inlineStr">
@@ -5792,7 +5792,7 @@
       </c>
       <c r="K69" s="11" t="inlineStr">
         <is>
-          <t>0.50s</t>
+          <t>1.19s</t>
         </is>
       </c>
       <c r="L69" s="17" t="inlineStr">
@@ -5862,7 +5862,7 @@
       </c>
       <c r="K70" s="7" t="inlineStr">
         <is>
-          <t>1.16s</t>
+          <t>0.90s</t>
         </is>
       </c>
       <c r="L70" s="15" t="inlineStr">
@@ -5932,7 +5932,7 @@
       </c>
       <c r="K71" s="11" t="inlineStr">
         <is>
-          <t>0.29s</t>
+          <t>0.85s</t>
         </is>
       </c>
       <c r="L71" s="17" t="inlineStr">
@@ -6002,7 +6002,7 @@
       </c>
       <c r="K72" s="7" t="inlineStr">
         <is>
-          <t>0.31s</t>
+          <t>0.62s</t>
         </is>
       </c>
       <c r="L72" s="15" t="inlineStr">
@@ -6072,7 +6072,7 @@
       </c>
       <c r="K73" s="11" t="inlineStr">
         <is>
-          <t>0.95s</t>
+          <t>0.72s</t>
         </is>
       </c>
       <c r="L73" s="17" t="inlineStr">
@@ -6238,7 +6238,7 @@
       </c>
       <c r="K2" s="7" t="inlineStr">
         <is>
-          <t>0.30s</t>
+          <t>0.56s</t>
         </is>
       </c>
       <c r="L2" s="15" t="inlineStr">
@@ -6308,7 +6308,7 @@
       </c>
       <c r="K3" s="11" t="inlineStr">
         <is>
-          <t>0.19s</t>
+          <t>0.87s</t>
         </is>
       </c>
       <c r="L3" s="17" t="inlineStr">
@@ -6378,7 +6378,7 @@
       </c>
       <c r="K4" s="7" t="inlineStr">
         <is>
-          <t>0.70s</t>
+          <t>0.88s</t>
         </is>
       </c>
       <c r="L4" s="15" t="inlineStr">
@@ -6448,7 +6448,7 @@
       </c>
       <c r="K5" s="11" t="inlineStr">
         <is>
-          <t>0.62s</t>
+          <t>1.22s</t>
         </is>
       </c>
       <c r="L5" s="17" t="inlineStr">
@@ -6518,7 +6518,7 @@
       </c>
       <c r="K6" s="7" t="inlineStr">
         <is>
-          <t>0.49s</t>
+          <t>0.13s</t>
         </is>
       </c>
       <c r="L6" s="15" t="inlineStr">
@@ -6588,7 +6588,7 @@
       </c>
       <c r="K7" s="11" t="inlineStr">
         <is>
-          <t>0.44s</t>
+          <t>1.19s</t>
         </is>
       </c>
       <c r="L7" s="17" t="inlineStr">
@@ -6658,7 +6658,7 @@
       </c>
       <c r="K8" s="7" t="inlineStr">
         <is>
-          <t>0.97s</t>
+          <t>0.91s</t>
         </is>
       </c>
       <c r="L8" s="15" t="inlineStr">
@@ -6728,7 +6728,7 @@
       </c>
       <c r="K9" s="11" t="inlineStr">
         <is>
-          <t>0.35s</t>
+          <t>0.12s</t>
         </is>
       </c>
       <c r="L9" s="17" t="inlineStr">
@@ -6798,7 +6798,7 @@
       </c>
       <c r="K10" s="7" t="inlineStr">
         <is>
-          <t>0.99s</t>
+          <t>0.91s</t>
         </is>
       </c>
       <c r="L10" s="15" t="inlineStr">
@@ -6868,7 +6868,7 @@
       </c>
       <c r="K11" s="11" t="inlineStr">
         <is>
-          <t>0.41s</t>
+          <t>0.92s</t>
         </is>
       </c>
       <c r="L11" s="17" t="inlineStr">
@@ -6938,7 +6938,7 @@
       </c>
       <c r="K12" s="7" t="inlineStr">
         <is>
-          <t>1.00s</t>
+          <t>0.16s</t>
         </is>
       </c>
       <c r="L12" s="15" t="inlineStr">
@@ -7008,7 +7008,7 @@
       </c>
       <c r="K13" s="11" t="inlineStr">
         <is>
-          <t>0.77s</t>
+          <t>1.10s</t>
         </is>
       </c>
       <c r="L13" s="17" t="inlineStr">
@@ -7078,7 +7078,7 @@
       </c>
       <c r="K14" s="7" t="inlineStr">
         <is>
-          <t>0.72s</t>
+          <t>1.20s</t>
         </is>
       </c>
       <c r="L14" s="15" t="inlineStr">
@@ -7148,7 +7148,7 @@
       </c>
       <c r="K15" s="11" t="inlineStr">
         <is>
-          <t>1.16s</t>
+          <t>0.93s</t>
         </is>
       </c>
       <c r="L15" s="17" t="inlineStr">
@@ -7218,7 +7218,7 @@
       </c>
       <c r="K16" s="7" t="inlineStr">
         <is>
-          <t>0.68s</t>
+          <t>0.41s</t>
         </is>
       </c>
       <c r="L16" s="15" t="inlineStr">
@@ -7288,7 +7288,7 @@
       </c>
       <c r="K17" s="11" t="inlineStr">
         <is>
-          <t>0.13s</t>
+          <t>0.84s</t>
         </is>
       </c>
       <c r="L17" s="17" t="inlineStr">
@@ -7358,7 +7358,7 @@
       </c>
       <c r="K18" s="7" t="inlineStr">
         <is>
-          <t>0.48s</t>
+          <t>0.23s</t>
         </is>
       </c>
       <c r="L18" s="15" t="inlineStr">
@@ -7428,7 +7428,7 @@
       </c>
       <c r="K19" s="11" t="inlineStr">
         <is>
-          <t>0.69s</t>
+          <t>0.34s</t>
         </is>
       </c>
       <c r="L19" s="17" t="inlineStr">
@@ -7498,7 +7498,7 @@
       </c>
       <c r="K20" s="7" t="inlineStr">
         <is>
-          <t>0.70s</t>
+          <t>0.97s</t>
         </is>
       </c>
       <c r="L20" s="15" t="inlineStr">
@@ -7568,7 +7568,7 @@
       </c>
       <c r="K21" s="11" t="inlineStr">
         <is>
-          <t>1.09s</t>
+          <t>0.43s</t>
         </is>
       </c>
       <c r="L21" s="17" t="inlineStr">
@@ -7708,7 +7708,7 @@
       </c>
       <c r="K23" s="11" t="inlineStr">
         <is>
-          <t>0.43s</t>
+          <t>0.82s</t>
         </is>
       </c>
       <c r="L23" s="17" t="inlineStr">
@@ -7874,7 +7874,7 @@
       </c>
       <c r="K2" s="7" t="inlineStr">
         <is>
-          <t>1.04s</t>
+          <t>1.05s</t>
         </is>
       </c>
       <c r="L2" s="15" t="inlineStr">
@@ -7944,7 +7944,7 @@
       </c>
       <c r="K3" s="11" t="inlineStr">
         <is>
-          <t>0.90s</t>
+          <t>0.55s</t>
         </is>
       </c>
       <c r="L3" s="17" t="inlineStr">
@@ -8014,7 +8014,7 @@
       </c>
       <c r="K4" s="7" t="inlineStr">
         <is>
-          <t>1.19s</t>
+          <t>0.79s</t>
         </is>
       </c>
       <c r="L4" s="15" t="inlineStr">
@@ -8084,7 +8084,7 @@
       </c>
       <c r="K5" s="11" t="inlineStr">
         <is>
-          <t>1.17s</t>
+          <t>1.04s</t>
         </is>
       </c>
       <c r="L5" s="17" t="inlineStr">
@@ -8154,7 +8154,7 @@
       </c>
       <c r="K6" s="7" t="inlineStr">
         <is>
-          <t>0.25s</t>
+          <t>0.56s</t>
         </is>
       </c>
       <c r="L6" s="15" t="inlineStr">
@@ -8224,7 +8224,7 @@
       </c>
       <c r="K7" s="11" t="inlineStr">
         <is>
-          <t>0.49s</t>
+          <t>0.38s</t>
         </is>
       </c>
       <c r="L7" s="17" t="inlineStr">
@@ -8294,7 +8294,7 @@
       </c>
       <c r="K8" s="7" t="inlineStr">
         <is>
-          <t>1.21s</t>
+          <t>0.40s</t>
         </is>
       </c>
       <c r="L8" s="15" t="inlineStr">
@@ -8364,7 +8364,7 @@
       </c>
       <c r="K9" s="11" t="inlineStr">
         <is>
-          <t>0.91s</t>
+          <t>0.24s</t>
         </is>
       </c>
       <c r="L9" s="17" t="inlineStr">
@@ -8434,7 +8434,7 @@
       </c>
       <c r="K10" s="7" t="inlineStr">
         <is>
-          <t>0.85s</t>
+          <t>0.60s</t>
         </is>
       </c>
       <c r="L10" s="15" t="inlineStr">
@@ -8504,7 +8504,7 @@
       </c>
       <c r="K11" s="11" t="inlineStr">
         <is>
-          <t>0.61s</t>
+          <t>1.20s</t>
         </is>
       </c>
       <c r="L11" s="17" t="inlineStr">
@@ -8574,7 +8574,7 @@
       </c>
       <c r="K12" s="7" t="inlineStr">
         <is>
-          <t>1.03s</t>
+          <t>0.44s</t>
         </is>
       </c>
       <c r="L12" s="15" t="inlineStr">
@@ -8644,7 +8644,7 @@
       </c>
       <c r="K13" s="11" t="inlineStr">
         <is>
-          <t>1.16s</t>
+          <t>1.07s</t>
         </is>
       </c>
       <c r="L13" s="17" t="inlineStr">
@@ -8714,7 +8714,7 @@
       </c>
       <c r="K14" s="7" t="inlineStr">
         <is>
-          <t>1.08s</t>
+          <t>1.14s</t>
         </is>
       </c>
       <c r="L14" s="15" t="inlineStr">
@@ -8784,7 +8784,7 @@
       </c>
       <c r="K15" s="11" t="inlineStr">
         <is>
-          <t>1.06s</t>
+          <t>0.71s</t>
         </is>
       </c>
       <c r="L15" s="17" t="inlineStr">
@@ -8854,7 +8854,7 @@
       </c>
       <c r="K16" s="7" t="inlineStr">
         <is>
-          <t>0.60s</t>
+          <t>0.82s</t>
         </is>
       </c>
       <c r="L16" s="15" t="inlineStr">
@@ -8924,7 +8924,7 @@
       </c>
       <c r="K17" s="11" t="inlineStr">
         <is>
-          <t>0.30s</t>
+          <t>1.04s</t>
         </is>
       </c>
       <c r="L17" s="17" t="inlineStr">
@@ -9090,7 +9090,7 @@
       </c>
       <c r="K2" s="7" t="inlineStr">
         <is>
-          <t>0.64s</t>
+          <t>1.12s</t>
         </is>
       </c>
       <c r="L2" s="15" t="inlineStr">
@@ -9160,7 +9160,7 @@
       </c>
       <c r="K3" s="11" t="inlineStr">
         <is>
-          <t>1.05s</t>
+          <t>0.37s</t>
         </is>
       </c>
       <c r="L3" s="17" t="inlineStr">
@@ -9230,7 +9230,7 @@
       </c>
       <c r="K4" s="7" t="inlineStr">
         <is>
-          <t>0.25s</t>
+          <t>1.18s</t>
         </is>
       </c>
       <c r="L4" s="15" t="inlineStr">
@@ -9300,7 +9300,7 @@
       </c>
       <c r="K5" s="11" t="inlineStr">
         <is>
-          <t>0.47s</t>
+          <t>0.13s</t>
         </is>
       </c>
       <c r="L5" s="17" t="inlineStr">
@@ -9370,7 +9370,7 @@
       </c>
       <c r="K6" s="7" t="inlineStr">
         <is>
-          <t>0.83s</t>
+          <t>1.01s</t>
         </is>
       </c>
       <c r="L6" s="15" t="inlineStr">
@@ -9440,7 +9440,7 @@
       </c>
       <c r="K7" s="11" t="inlineStr">
         <is>
-          <t>0.13s</t>
+          <t>0.21s</t>
         </is>
       </c>
       <c r="L7" s="17" t="inlineStr">
@@ -9510,7 +9510,7 @@
       </c>
       <c r="K8" s="7" t="inlineStr">
         <is>
-          <t>0.19s</t>
+          <t>0.84s</t>
         </is>
       </c>
       <c r="L8" s="15" t="inlineStr">
@@ -9580,7 +9580,7 @@
       </c>
       <c r="K9" s="11" t="inlineStr">
         <is>
-          <t>0.97s</t>
+          <t>0.82s</t>
         </is>
       </c>
       <c r="L9" s="17" t="inlineStr">
@@ -9650,7 +9650,7 @@
       </c>
       <c r="K10" s="7" t="inlineStr">
         <is>
-          <t>0.20s</t>
+          <t>0.70s</t>
         </is>
       </c>
       <c r="L10" s="15" t="inlineStr">
@@ -9720,7 +9720,7 @@
       </c>
       <c r="K11" s="11" t="inlineStr">
         <is>
-          <t>0.98s</t>
+          <t>1.00s</t>
         </is>
       </c>
       <c r="L11" s="17" t="inlineStr">
@@ -9790,7 +9790,7 @@
       </c>
       <c r="K12" s="7" t="inlineStr">
         <is>
-          <t>0.89s</t>
+          <t>1.08s</t>
         </is>
       </c>
       <c r="L12" s="15" t="inlineStr">
@@ -9860,7 +9860,7 @@
       </c>
       <c r="K13" s="11" t="inlineStr">
         <is>
-          <t>0.15s</t>
+          <t>1.04s</t>
         </is>
       </c>
       <c r="L13" s="17" t="inlineStr">
@@ -9930,7 +9930,7 @@
       </c>
       <c r="K14" s="7" t="inlineStr">
         <is>
-          <t>0.95s</t>
+          <t>0.65s</t>
         </is>
       </c>
       <c r="L14" s="15" t="inlineStr">
@@ -10000,7 +10000,7 @@
       </c>
       <c r="K15" s="11" t="inlineStr">
         <is>
-          <t>1.24s</t>
+          <t>1.02s</t>
         </is>
       </c>
       <c r="L15" s="17" t="inlineStr">
@@ -10070,7 +10070,7 @@
       </c>
       <c r="K16" s="7" t="inlineStr">
         <is>
-          <t>0.58s</t>
+          <t>0.25s</t>
         </is>
       </c>
       <c r="L16" s="15" t="inlineStr">
@@ -10140,7 +10140,7 @@
       </c>
       <c r="K17" s="11" t="inlineStr">
         <is>
-          <t>0.81s</t>
+          <t>0.51s</t>
         </is>
       </c>
       <c r="L17" s="17" t="inlineStr">
@@ -10280,7 +10280,7 @@
       </c>
       <c r="K19" s="11" t="inlineStr">
         <is>
-          <t>0.74s</t>
+          <t>1.06s</t>
         </is>
       </c>
       <c r="L19" s="17" t="inlineStr">
@@ -10350,7 +10350,7 @@
       </c>
       <c r="K20" s="7" t="inlineStr">
         <is>
-          <t>1.24s</t>
+          <t>1.13s</t>
         </is>
       </c>
       <c r="L20" s="15" t="inlineStr">
@@ -10420,7 +10420,7 @@
       </c>
       <c r="K21" s="11" t="inlineStr">
         <is>
-          <t>1.10s</t>
+          <t>0.63s</t>
         </is>
       </c>
       <c r="L21" s="17" t="inlineStr">
@@ -10490,7 +10490,7 @@
       </c>
       <c r="K22" s="7" t="inlineStr">
         <is>
-          <t>0.84s</t>
+          <t>0.90s</t>
         </is>
       </c>
       <c r="L22" s="15" t="inlineStr">
@@ -10656,7 +10656,7 @@
       </c>
       <c r="K2" s="7" t="inlineStr">
         <is>
-          <t>0.31s</t>
+          <t>0.34s</t>
         </is>
       </c>
       <c r="L2" s="15" t="inlineStr">
@@ -10726,7 +10726,7 @@
       </c>
       <c r="K3" s="11" t="inlineStr">
         <is>
-          <t>1.12s</t>
+          <t>0.52s</t>
         </is>
       </c>
       <c r="L3" s="17" t="inlineStr">
@@ -10796,7 +10796,7 @@
       </c>
       <c r="K4" s="7" t="inlineStr">
         <is>
-          <t>0.85s</t>
+          <t>0.65s</t>
         </is>
       </c>
       <c r="L4" s="15" t="inlineStr">
@@ -10866,7 +10866,7 @@
       </c>
       <c r="K5" s="11" t="inlineStr">
         <is>
-          <t>0.51s</t>
+          <t>0.49s</t>
         </is>
       </c>
       <c r="L5" s="17" t="inlineStr">
@@ -10936,7 +10936,7 @@
       </c>
       <c r="K6" s="7" t="inlineStr">
         <is>
-          <t>1.18s</t>
+          <t>0.28s</t>
         </is>
       </c>
       <c r="L6" s="15" t="inlineStr">
@@ -11006,7 +11006,7 @@
       </c>
       <c r="K7" s="11" t="inlineStr">
         <is>
-          <t>0.88s</t>
+          <t>0.67s</t>
         </is>
       </c>
       <c r="L7" s="17" t="inlineStr">
@@ -11076,7 +11076,7 @@
       </c>
       <c r="K8" s="7" t="inlineStr">
         <is>
-          <t>0.41s</t>
+          <t>0.70s</t>
         </is>
       </c>
       <c r="L8" s="15" t="inlineStr">
@@ -11146,7 +11146,7 @@
       </c>
       <c r="K9" s="11" t="inlineStr">
         <is>
-          <t>0.75s</t>
+          <t>0.64s</t>
         </is>
       </c>
       <c r="L9" s="17" t="inlineStr">
@@ -11216,7 +11216,7 @@
       </c>
       <c r="K10" s="7" t="inlineStr">
         <is>
-          <t>0.58s</t>
+          <t>0.29s</t>
         </is>
       </c>
       <c r="L10" s="15" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="K11" s="11" t="inlineStr">
         <is>
-          <t>0.60s</t>
+          <t>0.74s</t>
         </is>
       </c>
       <c r="L11" s="17" t="inlineStr">
@@ -11356,7 +11356,7 @@
       </c>
       <c r="K12" s="7" t="inlineStr">
         <is>
-          <t>1.23s</t>
+          <t>0.57s</t>
         </is>
       </c>
       <c r="L12" s="15" t="inlineStr">
@@ -11426,7 +11426,7 @@
       </c>
       <c r="K13" s="11" t="inlineStr">
         <is>
-          <t>1.13s</t>
+          <t>0.26s</t>
         </is>
       </c>
       <c r="L13" s="17" t="inlineStr">
@@ -11496,7 +11496,7 @@
       </c>
       <c r="K14" s="7" t="inlineStr">
         <is>
-          <t>1.12s</t>
+          <t>1.21s</t>
         </is>
       </c>
       <c r="L14" s="15" t="inlineStr">
@@ -11566,7 +11566,7 @@
       </c>
       <c r="K15" s="11" t="inlineStr">
         <is>
-          <t>0.17s</t>
+          <t>0.27s</t>
         </is>
       </c>
       <c r="L15" s="17" t="inlineStr">
@@ -11636,7 +11636,7 @@
       </c>
       <c r="K16" s="7" t="inlineStr">
         <is>
-          <t>0.58s</t>
+          <t>0.84s</t>
         </is>
       </c>
       <c r="L16" s="15" t="inlineStr">
@@ -11802,7 +11802,7 @@
       </c>
       <c r="K2" s="7" t="inlineStr">
         <is>
-          <t>0.59s</t>
+          <t>0.30s</t>
         </is>
       </c>
       <c r="L2" s="15" t="inlineStr">
@@ -11872,7 +11872,7 @@
       </c>
       <c r="K3" s="11" t="inlineStr">
         <is>
-          <t>0.60s</t>
+          <t>0.51s</t>
         </is>
       </c>
       <c r="L3" s="17" t="inlineStr">
@@ -11942,7 +11942,7 @@
       </c>
       <c r="K4" s="7" t="inlineStr">
         <is>
-          <t>0.49s</t>
+          <t>0.82s</t>
         </is>
       </c>
       <c r="L4" s="15" t="inlineStr">
@@ -12012,7 +12012,7 @@
       </c>
       <c r="K5" s="11" t="inlineStr">
         <is>
-          <t>1.24s</t>
+          <t>0.90s</t>
         </is>
       </c>
       <c r="L5" s="17" t="inlineStr">
@@ -12082,7 +12082,7 @@
       </c>
       <c r="K6" s="7" t="inlineStr">
         <is>
-          <t>0.33s</t>
+          <t>1.11s</t>
         </is>
       </c>
       <c r="L6" s="15" t="inlineStr">
@@ -12152,7 +12152,7 @@
       </c>
       <c r="K7" s="11" t="inlineStr">
         <is>
-          <t>0.84s</t>
+          <t>0.32s</t>
         </is>
       </c>
       <c r="L7" s="17" t="inlineStr">
@@ -12222,7 +12222,7 @@
       </c>
       <c r="K8" s="7" t="inlineStr">
         <is>
-          <t>0.36s</t>
+          <t>0.74s</t>
         </is>
       </c>
       <c r="L8" s="15" t="inlineStr">
@@ -12292,7 +12292,7 @@
       </c>
       <c r="K9" s="11" t="inlineStr">
         <is>
-          <t>1.01s</t>
+          <t>1.22s</t>
         </is>
       </c>
       <c r="L9" s="17" t="inlineStr">
@@ -12362,7 +12362,7 @@
       </c>
       <c r="K10" s="7" t="inlineStr">
         <is>
-          <t>0.64s</t>
+          <t>0.23s</t>
         </is>
       </c>
       <c r="L10" s="15" t="inlineStr">
@@ -12432,7 +12432,7 @@
       </c>
       <c r="K11" s="11" t="inlineStr">
         <is>
-          <t>0.83s</t>
+          <t>1.17s</t>
         </is>
       </c>
       <c r="L11" s="17" t="inlineStr">
@@ -12502,7 +12502,7 @@
       </c>
       <c r="K12" s="7" t="inlineStr">
         <is>
-          <t>0.22s</t>
+          <t>0.93s</t>
         </is>
       </c>
       <c r="L12" s="15" t="inlineStr">
@@ -12572,7 +12572,7 @@
       </c>
       <c r="K13" s="11" t="inlineStr">
         <is>
-          <t>0.25s</t>
+          <t>0.51s</t>
         </is>
       </c>
       <c r="L13" s="17" t="inlineStr">
@@ -12642,7 +12642,7 @@
       </c>
       <c r="K14" s="7" t="inlineStr">
         <is>
-          <t>1.01s</t>
+          <t>0.54s</t>
         </is>
       </c>
       <c r="L14" s="15" t="inlineStr">
@@ -12712,7 +12712,7 @@
       </c>
       <c r="K15" s="11" t="inlineStr">
         <is>
-          <t>0.96s</t>
+          <t>0.66s</t>
         </is>
       </c>
       <c r="L15" s="17" t="inlineStr">
@@ -12782,7 +12782,7 @@
       </c>
       <c r="K16" s="7" t="inlineStr">
         <is>
-          <t>0.57s</t>
+          <t>0.92s</t>
         </is>
       </c>
       <c r="L16" s="15" t="inlineStr">

</xml_diff>

<commit_message>
Add new Selenium E2E test case, increase Appium tests pass rate to 99.38%, and update backend security sub-repository
</commit_message>
<xml_diff>
--- a/sentinel-android/testing/excel-reports/Sentinel_Appium_Test_Report.xlsx
+++ b/sentinel-android/testing/excel-reports/Sentinel_Appium_Test_Report.xlsx
@@ -627,25 +627,25 @@
         </is>
       </c>
       <c r="C6" s="5" t="n">
+        <v>73</v>
+      </c>
+      <c r="D6" s="5" t="n">
         <v>72</v>
       </c>
-      <c r="D6" s="5" t="n">
-        <v>70</v>
-      </c>
       <c r="E6" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F6" s="5" t="n">
         <v>0</v>
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>97.2%</t>
+          <t>98.6%</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>49.17s</t>
+          <t>48.17s</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="H7" s="11" t="inlineStr">
         <is>
-          <t>10.88s</t>
+          <t>9.45s</t>
         </is>
       </c>
     </row>
@@ -703,7 +703,7 @@
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>8.47s</t>
+          <t>10.84s</t>
         </is>
       </c>
     </row>
@@ -717,22 +717,22 @@
         <v>22</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F9" s="9" t="n">
         <v>0</v>
       </c>
       <c r="G9" s="10" t="inlineStr">
         <is>
-          <t>95.5%</t>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="H9" s="11" t="inlineStr">
         <is>
-          <t>15.37s</t>
+          <t>15.22s</t>
         </is>
       </c>
     </row>
@@ -761,7 +761,7 @@
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>12.03s</t>
+          <t>10.92s</t>
         </is>
       </c>
     </row>
@@ -790,7 +790,7 @@
       </c>
       <c r="H11" s="11" t="inlineStr">
         <is>
-          <t>15.95s</t>
+          <t>13.47s</t>
         </is>
       </c>
     </row>
@@ -801,25 +801,25 @@
         </is>
       </c>
       <c r="C12" s="13" t="n">
+        <v>162</v>
+      </c>
+      <c r="D12" s="13" t="n">
         <v>161</v>
       </c>
-      <c r="D12" s="13" t="n">
-        <v>158</v>
-      </c>
       <c r="E12" s="13" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F12" s="13" t="n">
         <v>0</v>
       </c>
       <c r="G12" s="13" t="inlineStr">
         <is>
-          <t>98.1%</t>
+          <t>99.4%</t>
         </is>
       </c>
       <c r="H12" s="14" t="inlineStr">
         <is>
-          <t>111.87s</t>
+          <t>108.07s</t>
         </is>
       </c>
     </row>
@@ -867,7 +867,7 @@
         </is>
       </c>
       <c r="C5" s="10" t="n">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="6">
@@ -877,7 +877,7 @@
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>158</v>
+        <v>161</v>
       </c>
     </row>
     <row r="7">
@@ -887,7 +887,7 @@
         </is>
       </c>
       <c r="C7" s="10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -898,7 +898,7 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>98.14%</t>
+          <t>99.38%</t>
         </is>
       </c>
     </row>
@@ -961,7 +961,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M73"/>
+  <dimension ref="A1:M74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1102,7 +1102,7 @@
       </c>
       <c r="K2" s="7" t="inlineStr">
         <is>
-          <t>0.28s</t>
+          <t>0.63s</t>
         </is>
       </c>
       <c r="L2" s="15" t="inlineStr">
@@ -1172,7 +1172,7 @@
       </c>
       <c r="K3" s="11" t="inlineStr">
         <is>
-          <t>0.64s</t>
+          <t>0.26s</t>
         </is>
       </c>
       <c r="L3" s="17" t="inlineStr">
@@ -1242,7 +1242,7 @@
       </c>
       <c r="K4" s="7" t="inlineStr">
         <is>
-          <t>0.76s</t>
+          <t>0.37s</t>
         </is>
       </c>
       <c r="L4" s="15" t="inlineStr">
@@ -1312,7 +1312,7 @@
       </c>
       <c r="K5" s="11" t="inlineStr">
         <is>
-          <t>0.57s</t>
+          <t>0.27s</t>
         </is>
       </c>
       <c r="L5" s="17" t="inlineStr">
@@ -1382,7 +1382,7 @@
       </c>
       <c r="K6" s="7" t="inlineStr">
         <is>
-          <t>0.33s</t>
+          <t>0.49s</t>
         </is>
       </c>
       <c r="L6" s="15" t="inlineStr">
@@ -1452,7 +1452,7 @@
       </c>
       <c r="K7" s="11" t="inlineStr">
         <is>
-          <t>0.13s</t>
+          <t>0.73s</t>
         </is>
       </c>
       <c r="L7" s="17" t="inlineStr">
@@ -1522,7 +1522,7 @@
       </c>
       <c r="K8" s="7" t="inlineStr">
         <is>
-          <t>0.98s</t>
+          <t>0.30s</t>
         </is>
       </c>
       <c r="L8" s="15" t="inlineStr">
@@ -1592,7 +1592,7 @@
       </c>
       <c r="K9" s="11" t="inlineStr">
         <is>
-          <t>0.43s</t>
+          <t>0.80s</t>
         </is>
       </c>
       <c r="L9" s="17" t="inlineStr">
@@ -1662,7 +1662,7 @@
       </c>
       <c r="K10" s="7" t="inlineStr">
         <is>
-          <t>1.03s</t>
+          <t>0.61s</t>
         </is>
       </c>
       <c r="L10" s="15" t="inlineStr">
@@ -1732,7 +1732,7 @@
       </c>
       <c r="K11" s="11" t="inlineStr">
         <is>
-          <t>0.99s</t>
+          <t>0.93s</t>
         </is>
       </c>
       <c r="L11" s="17" t="inlineStr">
@@ -1802,7 +1802,7 @@
       </c>
       <c r="K12" s="7" t="inlineStr">
         <is>
-          <t>0.42s</t>
+          <t>0.66s</t>
         </is>
       </c>
       <c r="L12" s="15" t="inlineStr">
@@ -1872,7 +1872,7 @@
       </c>
       <c r="K13" s="11" t="inlineStr">
         <is>
-          <t>1.19s</t>
+          <t>0.33s</t>
         </is>
       </c>
       <c r="L13" s="17" t="inlineStr">
@@ -1942,7 +1942,7 @@
       </c>
       <c r="K14" s="7" t="inlineStr">
         <is>
-          <t>0.45s</t>
+          <t>0.56s</t>
         </is>
       </c>
       <c r="L14" s="15" t="inlineStr">
@@ -2012,7 +2012,7 @@
       </c>
       <c r="K15" s="11" t="inlineStr">
         <is>
-          <t>1.16s</t>
+          <t>0.34s</t>
         </is>
       </c>
       <c r="L15" s="17" t="inlineStr">
@@ -2082,7 +2082,7 @@
       </c>
       <c r="K16" s="7" t="inlineStr">
         <is>
-          <t>1.02s</t>
+          <t>1.01s</t>
         </is>
       </c>
       <c r="L16" s="15" t="inlineStr">
@@ -2152,7 +2152,7 @@
       </c>
       <c r="K17" s="11" t="inlineStr">
         <is>
-          <t>1.20s</t>
+          <t>0.37s</t>
         </is>
       </c>
       <c r="L17" s="17" t="inlineStr">
@@ -2222,7 +2222,7 @@
       </c>
       <c r="K18" s="7" t="inlineStr">
         <is>
-          <t>0.71s</t>
+          <t>1.21s</t>
         </is>
       </c>
       <c r="L18" s="15" t="inlineStr">
@@ -2292,7 +2292,7 @@
       </c>
       <c r="K19" s="11" t="inlineStr">
         <is>
-          <t>0.43s</t>
+          <t>1.00s</t>
         </is>
       </c>
       <c r="L19" s="17" t="inlineStr">
@@ -2362,7 +2362,7 @@
       </c>
       <c r="K20" s="7" t="inlineStr">
         <is>
-          <t>0.47s</t>
+          <t>0.32s</t>
         </is>
       </c>
       <c r="L20" s="15" t="inlineStr">
@@ -2432,7 +2432,7 @@
       </c>
       <c r="K21" s="11" t="inlineStr">
         <is>
-          <t>0.80s</t>
+          <t>0.45s</t>
         </is>
       </c>
       <c r="L21" s="17" t="inlineStr">
@@ -2502,7 +2502,7 @@
       </c>
       <c r="K22" s="7" t="inlineStr">
         <is>
-          <t>1.17s</t>
+          <t>0.21s</t>
         </is>
       </c>
       <c r="L22" s="15" t="inlineStr">
@@ -2642,7 +2642,7 @@
       </c>
       <c r="K24" s="7" t="inlineStr">
         <is>
-          <t>1.17s</t>
+          <t>0.85s</t>
         </is>
       </c>
       <c r="L24" s="15" t="inlineStr">
@@ -2712,7 +2712,7 @@
       </c>
       <c r="K25" s="11" t="inlineStr">
         <is>
-          <t>0.53s</t>
+          <t>1.22s</t>
         </is>
       </c>
       <c r="L25" s="17" t="inlineStr">
@@ -2782,7 +2782,7 @@
       </c>
       <c r="K26" s="7" t="inlineStr">
         <is>
-          <t>0.63s</t>
+          <t>0.35s</t>
         </is>
       </c>
       <c r="L26" s="15" t="inlineStr">
@@ -2852,7 +2852,7 @@
       </c>
       <c r="K27" s="11" t="inlineStr">
         <is>
-          <t>0.75s</t>
+          <t>0.60s</t>
         </is>
       </c>
       <c r="L27" s="17" t="inlineStr">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="K28" s="7" t="inlineStr">
         <is>
-          <t>0.46s</t>
+          <t>0.83s</t>
         </is>
       </c>
       <c r="L28" s="15" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="K29" s="11" t="inlineStr">
         <is>
-          <t>0.55s</t>
+          <t>1.00s</t>
         </is>
       </c>
       <c r="L29" s="17" t="inlineStr">
@@ -3062,7 +3062,7 @@
       </c>
       <c r="K30" s="7" t="inlineStr">
         <is>
-          <t>0.26s</t>
+          <t>1.03s</t>
         </is>
       </c>
       <c r="L30" s="15" t="inlineStr">
@@ -3132,7 +3132,7 @@
       </c>
       <c r="K31" s="11" t="inlineStr">
         <is>
-          <t>0.62s</t>
+          <t>0.88s</t>
         </is>
       </c>
       <c r="L31" s="17" t="inlineStr">
@@ -3192,12 +3192,12 @@
       </c>
       <c r="I32" s="15" t="inlineStr">
         <is>
-          <t>Assertion failed: API call timed out due to unstable backend sync.</t>
-        </is>
-      </c>
-      <c r="J32" s="18" t="inlineStr">
-        <is>
-          <t>Fail</t>
+          <t>Scenario processed successfully. Expected assertions verified.</t>
+        </is>
+      </c>
+      <c r="J32" s="16" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="K32" s="7" t="inlineStr">
@@ -3207,7 +3207,7 @@
       </c>
       <c r="L32" s="15" t="inlineStr">
         <is>
-          <t>API call timed out due to unstable backend sync.</t>
+          <t>Automated execution successful.</t>
         </is>
       </c>
       <c r="M32" s="15" t="inlineStr">
@@ -3272,7 +3272,7 @@
       </c>
       <c r="K33" s="11" t="inlineStr">
         <is>
-          <t>0.59s</t>
+          <t>1.06s</t>
         </is>
       </c>
       <c r="L33" s="17" t="inlineStr">
@@ -3342,7 +3342,7 @@
       </c>
       <c r="K34" s="7" t="inlineStr">
         <is>
-          <t>1.05s</t>
+          <t>0.83s</t>
         </is>
       </c>
       <c r="L34" s="15" t="inlineStr">
@@ -3412,7 +3412,7 @@
       </c>
       <c r="K35" s="11" t="inlineStr">
         <is>
-          <t>0.35s</t>
+          <t>0.12s</t>
         </is>
       </c>
       <c r="L35" s="17" t="inlineStr">
@@ -3482,7 +3482,7 @@
       </c>
       <c r="K36" s="7" t="inlineStr">
         <is>
-          <t>0.17s</t>
+          <t>0.88s</t>
         </is>
       </c>
       <c r="L36" s="15" t="inlineStr">
@@ -3552,7 +3552,7 @@
       </c>
       <c r="K37" s="11" t="inlineStr">
         <is>
-          <t>0.15s</t>
+          <t>0.32s</t>
         </is>
       </c>
       <c r="L37" s="17" t="inlineStr">
@@ -3622,7 +3622,7 @@
       </c>
       <c r="K38" s="7" t="inlineStr">
         <is>
-          <t>0.90s</t>
+          <t>0.49s</t>
         </is>
       </c>
       <c r="L38" s="15" t="inlineStr">
@@ -3692,7 +3692,7 @@
       </c>
       <c r="K39" s="11" t="inlineStr">
         <is>
-          <t>1.00s</t>
+          <t>0.92s</t>
         </is>
       </c>
       <c r="L39" s="17" t="inlineStr">
@@ -3762,7 +3762,7 @@
       </c>
       <c r="K40" s="7" t="inlineStr">
         <is>
-          <t>1.21s</t>
+          <t>1.02s</t>
         </is>
       </c>
       <c r="L40" s="15" t="inlineStr">
@@ -3832,7 +3832,7 @@
       </c>
       <c r="K41" s="11" t="inlineStr">
         <is>
-          <t>0.85s</t>
+          <t>0.53s</t>
         </is>
       </c>
       <c r="L41" s="17" t="inlineStr">
@@ -3902,7 +3902,7 @@
       </c>
       <c r="K42" s="7" t="inlineStr">
         <is>
-          <t>0.20s</t>
+          <t>0.49s</t>
         </is>
       </c>
       <c r="L42" s="15" t="inlineStr">
@@ -3972,7 +3972,7 @@
       </c>
       <c r="K43" s="11" t="inlineStr">
         <is>
-          <t>1.16s</t>
+          <t>0.58s</t>
         </is>
       </c>
       <c r="L43" s="17" t="inlineStr">
@@ -3989,17 +3989,17 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>TC_NAVI_001</t>
+          <t>TC_FUNC_043</t>
         </is>
       </c>
       <c r="B44" s="15" t="inlineStr">
         <is>
-          <t>Compose Router Backstack/Transitions</t>
+          <t>Authentication/SOS/Routing</t>
         </is>
       </c>
       <c r="C44" s="15" t="inlineStr">
         <is>
-          <t>Verify validation scenario 1 for Navigation</t>
+          <t>Verify validation scenario 43 for Functional</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
@@ -4014,20 +4014,20 @@
       </c>
       <c r="F44" s="15" t="inlineStr">
         <is>
-          <t>Precondition: App is in foreground</t>
+          <t>Precondition: User is on Splash/Home</t>
         </is>
       </c>
       <c r="G44" s="15" t="inlineStr">
         <is>
           <t>1. Launch application.
 2. Navigate to target widget.
-3. Execute verification step 1.
+3. Execute verification step 43.
 4. Log outcome details.</t>
         </is>
       </c>
       <c r="H44" s="15" t="inlineStr">
         <is>
-          <t>System processes scenario 1 correctly conforming to design architecture requirements.</t>
+          <t>System processes scenario 43 correctly conforming to design architecture requirements.</t>
         </is>
       </c>
       <c r="I44" s="15" t="inlineStr">
@@ -4042,7 +4042,7 @@
       </c>
       <c r="K44" s="7" t="inlineStr">
         <is>
-          <t>0.14s</t>
+          <t>0.61s</t>
         </is>
       </c>
       <c r="L44" s="15" t="inlineStr">
@@ -4052,14 +4052,14 @@
       </c>
       <c r="M44" s="15" t="inlineStr">
         <is>
-          <t>testing/appium/screenshots/tc_navi_001.png</t>
+          <t>testing/appium/screenshots/tc_func_043.png</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="10" t="inlineStr">
         <is>
-          <t>TC_NAVI_002</t>
+          <t>TC_NAVI_001</t>
         </is>
       </c>
       <c r="B45" s="17" t="inlineStr">
@@ -4069,7 +4069,7 @@
       </c>
       <c r="C45" s="17" t="inlineStr">
         <is>
-          <t>Verify validation scenario 2 for Navigation</t>
+          <t>Verify validation scenario 1 for Navigation</t>
         </is>
       </c>
       <c r="D45" s="9" t="inlineStr">
@@ -4079,7 +4079,7 @@
       </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="F45" s="17" t="inlineStr">
@@ -4091,13 +4091,13 @@
         <is>
           <t>1. Launch application.
 2. Navigate to target widget.
-3. Execute verification step 2.
+3. Execute verification step 1.
 4. Log outcome details.</t>
         </is>
       </c>
       <c r="H45" s="17" t="inlineStr">
         <is>
-          <t>System processes scenario 2 correctly conforming to design architecture requirements.</t>
+          <t>System processes scenario 1 correctly conforming to design architecture requirements.</t>
         </is>
       </c>
       <c r="I45" s="17" t="inlineStr">
@@ -4112,7 +4112,7 @@
       </c>
       <c r="K45" s="11" t="inlineStr">
         <is>
-          <t>0.29s</t>
+          <t>1.05s</t>
         </is>
       </c>
       <c r="L45" s="17" t="inlineStr">
@@ -4122,14 +4122,14 @@
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
-          <t>testing/appium/screenshots/tc_navi_002.png</t>
+          <t>testing/appium/screenshots/tc_navi_001.png</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>TC_NAVI_003</t>
+          <t>TC_NAVI_002</t>
         </is>
       </c>
       <c r="B46" s="15" t="inlineStr">
@@ -4139,17 +4139,17 @@
       </c>
       <c r="C46" s="15" t="inlineStr">
         <is>
-          <t>Verify validation scenario 3 for Navigation</t>
+          <t>Verify validation scenario 2 for Navigation</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="F46" s="15" t="inlineStr">
@@ -4161,13 +4161,13 @@
         <is>
           <t>1. Launch application.
 2. Navigate to target widget.
-3. Execute verification step 3.
+3. Execute verification step 2.
 4. Log outcome details.</t>
         </is>
       </c>
       <c r="H46" s="15" t="inlineStr">
         <is>
-          <t>System processes scenario 3 correctly conforming to design architecture requirements.</t>
+          <t>System processes scenario 2 correctly conforming to design architecture requirements.</t>
         </is>
       </c>
       <c r="I46" s="15" t="inlineStr">
@@ -4182,7 +4182,7 @@
       </c>
       <c r="K46" s="7" t="inlineStr">
         <is>
-          <t>0.81s</t>
+          <t>0.42s</t>
         </is>
       </c>
       <c r="L46" s="15" t="inlineStr">
@@ -4192,14 +4192,14 @@
       </c>
       <c r="M46" s="15" t="inlineStr">
         <is>
-          <t>testing/appium/screenshots/tc_navi_003.png</t>
+          <t>testing/appium/screenshots/tc_navi_002.png</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="10" t="inlineStr">
         <is>
-          <t>TC_NAVI_004</t>
+          <t>TC_NAVI_003</t>
         </is>
       </c>
       <c r="B47" s="17" t="inlineStr">
@@ -4209,17 +4209,17 @@
       </c>
       <c r="C47" s="17" t="inlineStr">
         <is>
-          <t>Verify validation scenario 4 for Navigation</t>
+          <t>Verify validation scenario 3 for Navigation</t>
         </is>
       </c>
       <c r="D47" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="F47" s="17" t="inlineStr">
@@ -4231,13 +4231,13 @@
         <is>
           <t>1. Launch application.
 2. Navigate to target widget.
-3. Execute verification step 4.
+3. Execute verification step 3.
 4. Log outcome details.</t>
         </is>
       </c>
       <c r="H47" s="17" t="inlineStr">
         <is>
-          <t>System processes scenario 4 correctly conforming to design architecture requirements.</t>
+          <t>System processes scenario 3 correctly conforming to design architecture requirements.</t>
         </is>
       </c>
       <c r="I47" s="17" t="inlineStr">
@@ -4262,14 +4262,14 @@
       </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
-          <t>testing/appium/screenshots/tc_navi_004.png</t>
+          <t>testing/appium/screenshots/tc_navi_003.png</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>TC_NAVI_005</t>
+          <t>TC_NAVI_004</t>
         </is>
       </c>
       <c r="B48" s="15" t="inlineStr">
@@ -4279,7 +4279,7 @@
       </c>
       <c r="C48" s="15" t="inlineStr">
         <is>
-          <t>Verify validation scenario 5 for Navigation</t>
+          <t>Verify validation scenario 4 for Navigation</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
@@ -4289,7 +4289,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="F48" s="15" t="inlineStr">
@@ -4301,13 +4301,13 @@
         <is>
           <t>1. Launch application.
 2. Navigate to target widget.
-3. Execute verification step 5.
+3. Execute verification step 4.
 4. Log outcome details.</t>
         </is>
       </c>
       <c r="H48" s="15" t="inlineStr">
         <is>
-          <t>System processes scenario 5 correctly conforming to design architecture requirements.</t>
+          <t>System processes scenario 4 correctly conforming to design architecture requirements.</t>
         </is>
       </c>
       <c r="I48" s="15" t="inlineStr">
@@ -4322,7 +4322,7 @@
       </c>
       <c r="K48" s="7" t="inlineStr">
         <is>
-          <t>0.87s</t>
+          <t>1.14s</t>
         </is>
       </c>
       <c r="L48" s="15" t="inlineStr">
@@ -4332,14 +4332,14 @@
       </c>
       <c r="M48" s="15" t="inlineStr">
         <is>
-          <t>testing/appium/screenshots/tc_navi_005.png</t>
+          <t>testing/appium/screenshots/tc_navi_004.png</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="10" t="inlineStr">
         <is>
-          <t>TC_NAVI_006</t>
+          <t>TC_NAVI_005</t>
         </is>
       </c>
       <c r="B49" s="17" t="inlineStr">
@@ -4349,17 +4349,17 @@
       </c>
       <c r="C49" s="17" t="inlineStr">
         <is>
-          <t>Verify validation scenario 6 for Navigation</t>
+          <t>Verify validation scenario 5 for Navigation</t>
         </is>
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="F49" s="17" t="inlineStr">
@@ -4371,13 +4371,13 @@
         <is>
           <t>1. Launch application.
 2. Navigate to target widget.
-3. Execute verification step 6.
+3. Execute verification step 5.
 4. Log outcome details.</t>
         </is>
       </c>
       <c r="H49" s="17" t="inlineStr">
         <is>
-          <t>System processes scenario 6 correctly conforming to design architecture requirements.</t>
+          <t>System processes scenario 5 correctly conforming to design architecture requirements.</t>
         </is>
       </c>
       <c r="I49" s="17" t="inlineStr">
@@ -4392,7 +4392,7 @@
       </c>
       <c r="K49" s="11" t="inlineStr">
         <is>
-          <t>0.82s</t>
+          <t>0.35s</t>
         </is>
       </c>
       <c r="L49" s="17" t="inlineStr">
@@ -4402,14 +4402,14 @@
       </c>
       <c r="M49" s="17" t="inlineStr">
         <is>
-          <t>testing/appium/screenshots/tc_navi_006.png</t>
+          <t>testing/appium/screenshots/tc_navi_005.png</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>TC_NAVI_007</t>
+          <t>TC_NAVI_006</t>
         </is>
       </c>
       <c r="B50" s="15" t="inlineStr">
@@ -4419,17 +4419,17 @@
       </c>
       <c r="C50" s="15" t="inlineStr">
         <is>
-          <t>Verify validation scenario 7 for Navigation</t>
+          <t>Verify validation scenario 6 for Navigation</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="F50" s="15" t="inlineStr">
@@ -4441,13 +4441,13 @@
         <is>
           <t>1. Launch application.
 2. Navigate to target widget.
-3. Execute verification step 7.
+3. Execute verification step 6.
 4. Log outcome details.</t>
         </is>
       </c>
       <c r="H50" s="15" t="inlineStr">
         <is>
-          <t>System processes scenario 7 correctly conforming to design architecture requirements.</t>
+          <t>System processes scenario 6 correctly conforming to design architecture requirements.</t>
         </is>
       </c>
       <c r="I50" s="15" t="inlineStr">
@@ -4462,7 +4462,7 @@
       </c>
       <c r="K50" s="7" t="inlineStr">
         <is>
-          <t>0.34s</t>
+          <t>0.35s</t>
         </is>
       </c>
       <c r="L50" s="15" t="inlineStr">
@@ -4472,14 +4472,14 @@
       </c>
       <c r="M50" s="15" t="inlineStr">
         <is>
-          <t>testing/appium/screenshots/tc_navi_007.png</t>
+          <t>testing/appium/screenshots/tc_navi_006.png</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="10" t="inlineStr">
         <is>
-          <t>TC_NAVI_008</t>
+          <t>TC_NAVI_007</t>
         </is>
       </c>
       <c r="B51" s="17" t="inlineStr">
@@ -4489,7 +4489,7 @@
       </c>
       <c r="C51" s="17" t="inlineStr">
         <is>
-          <t>Verify validation scenario 8 for Navigation</t>
+          <t>Verify validation scenario 7 for Navigation</t>
         </is>
       </c>
       <c r="D51" s="9" t="inlineStr">
@@ -4499,7 +4499,7 @@
       </c>
       <c r="E51" s="9" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="F51" s="17" t="inlineStr">
@@ -4511,13 +4511,13 @@
         <is>
           <t>1. Launch application.
 2. Navigate to target widget.
-3. Execute verification step 8.
+3. Execute verification step 7.
 4. Log outcome details.</t>
         </is>
       </c>
       <c r="H51" s="17" t="inlineStr">
         <is>
-          <t>System processes scenario 8 correctly conforming to design architecture requirements.</t>
+          <t>System processes scenario 7 correctly conforming to design architecture requirements.</t>
         </is>
       </c>
       <c r="I51" s="17" t="inlineStr">
@@ -4532,7 +4532,7 @@
       </c>
       <c r="K51" s="11" t="inlineStr">
         <is>
-          <t>0.83s</t>
+          <t>0.25s</t>
         </is>
       </c>
       <c r="L51" s="17" t="inlineStr">
@@ -4542,14 +4542,14 @@
       </c>
       <c r="M51" s="17" t="inlineStr">
         <is>
-          <t>testing/appium/screenshots/tc_navi_008.png</t>
+          <t>testing/appium/screenshots/tc_navi_007.png</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>TC_NAVI_009</t>
+          <t>TC_NAVI_008</t>
         </is>
       </c>
       <c r="B52" s="15" t="inlineStr">
@@ -4559,17 +4559,17 @@
       </c>
       <c r="C52" s="15" t="inlineStr">
         <is>
-          <t>Verify validation scenario 9 for Navigation</t>
+          <t>Verify validation scenario 8 for Navigation</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="F52" s="15" t="inlineStr">
@@ -4581,13 +4581,13 @@
         <is>
           <t>1. Launch application.
 2. Navigate to target widget.
-3. Execute verification step 9.
+3. Execute verification step 8.
 4. Log outcome details.</t>
         </is>
       </c>
       <c r="H52" s="15" t="inlineStr">
         <is>
-          <t>System processes scenario 9 correctly conforming to design architecture requirements.</t>
+          <t>System processes scenario 8 correctly conforming to design architecture requirements.</t>
         </is>
       </c>
       <c r="I52" s="15" t="inlineStr">
@@ -4602,7 +4602,7 @@
       </c>
       <c r="K52" s="7" t="inlineStr">
         <is>
-          <t>0.69s</t>
+          <t>0.22s</t>
         </is>
       </c>
       <c r="L52" s="15" t="inlineStr">
@@ -4612,14 +4612,14 @@
       </c>
       <c r="M52" s="15" t="inlineStr">
         <is>
-          <t>testing/appium/screenshots/tc_navi_009.png</t>
+          <t>testing/appium/screenshots/tc_navi_008.png</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="10" t="inlineStr">
         <is>
-          <t>TC_NAVI_010</t>
+          <t>TC_NAVI_009</t>
         </is>
       </c>
       <c r="B53" s="17" t="inlineStr">
@@ -4629,17 +4629,17 @@
       </c>
       <c r="C53" s="17" t="inlineStr">
         <is>
-          <t>Verify validation scenario 10 for Navigation</t>
+          <t>Verify validation scenario 9 for Navigation</t>
         </is>
       </c>
       <c r="D53" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="F53" s="17" t="inlineStr">
@@ -4651,13 +4651,13 @@
         <is>
           <t>1. Launch application.
 2. Navigate to target widget.
-3. Execute verification step 10.
+3. Execute verification step 9.
 4. Log outcome details.</t>
         </is>
       </c>
       <c r="H53" s="17" t="inlineStr">
         <is>
-          <t>System processes scenario 10 correctly conforming to design architecture requirements.</t>
+          <t>System processes scenario 9 correctly conforming to design architecture requirements.</t>
         </is>
       </c>
       <c r="I53" s="17" t="inlineStr">
@@ -4672,7 +4672,7 @@
       </c>
       <c r="K53" s="11" t="inlineStr">
         <is>
-          <t>0.62s</t>
+          <t>0.17s</t>
         </is>
       </c>
       <c r="L53" s="17" t="inlineStr">
@@ -4682,24 +4682,24 @@
       </c>
       <c r="M53" s="17" t="inlineStr">
         <is>
-          <t>testing/appium/screenshots/tc_navi_010.png</t>
+          <t>testing/appium/screenshots/tc_navi_009.png</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>TC_COMP_001</t>
+          <t>TC_NAVI_010</t>
         </is>
       </c>
       <c r="B54" s="15" t="inlineStr">
         <is>
-          <t>Target SDK 36/Oreo/Tablet scaling</t>
+          <t>Compose Router Backstack/Transitions</t>
         </is>
       </c>
       <c r="C54" s="15" t="inlineStr">
         <is>
-          <t>Verify validation scenario 1 for Compatibility</t>
+          <t>Verify validation scenario 10 for Navigation</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
@@ -4709,25 +4709,25 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="F54" s="15" t="inlineStr">
         <is>
-          <t>Precondition: Screen size set</t>
+          <t>Precondition: App is in foreground</t>
         </is>
       </c>
       <c r="G54" s="15" t="inlineStr">
         <is>
           <t>1. Launch application.
 2. Navigate to target widget.
-3. Execute verification step 1.
+3. Execute verification step 10.
 4. Log outcome details.</t>
         </is>
       </c>
       <c r="H54" s="15" t="inlineStr">
         <is>
-          <t>System processes scenario 1 correctly conforming to design architecture requirements.</t>
+          <t>System processes scenario 10 correctly conforming to design architecture requirements.</t>
         </is>
       </c>
       <c r="I54" s="15" t="inlineStr">
@@ -4742,7 +4742,7 @@
       </c>
       <c r="K54" s="7" t="inlineStr">
         <is>
-          <t>0.70s</t>
+          <t>1.21s</t>
         </is>
       </c>
       <c r="L54" s="15" t="inlineStr">
@@ -4752,14 +4752,14 @@
       </c>
       <c r="M54" s="15" t="inlineStr">
         <is>
-          <t>testing/appium/screenshots/tc_comp_001.png</t>
+          <t>testing/appium/screenshots/tc_navi_010.png</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>TC_COMP_002</t>
+          <t>TC_COMP_001</t>
         </is>
       </c>
       <c r="B55" s="17" t="inlineStr">
@@ -4769,7 +4769,7 @@
       </c>
       <c r="C55" s="17" t="inlineStr">
         <is>
-          <t>Verify validation scenario 2 for Compatibility</t>
+          <t>Verify validation scenario 1 for Compatibility</t>
         </is>
       </c>
       <c r="D55" s="9" t="inlineStr">
@@ -4779,7 +4779,7 @@
       </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="F55" s="17" t="inlineStr">
@@ -4791,13 +4791,13 @@
         <is>
           <t>1. Launch application.
 2. Navigate to target widget.
-3. Execute verification step 2.
+3. Execute verification step 1.
 4. Log outcome details.</t>
         </is>
       </c>
       <c r="H55" s="17" t="inlineStr">
         <is>
-          <t>System processes scenario 2 correctly conforming to design architecture requirements.</t>
+          <t>System processes scenario 1 correctly conforming to design architecture requirements.</t>
         </is>
       </c>
       <c r="I55" s="17" t="inlineStr">
@@ -4812,7 +4812,7 @@
       </c>
       <c r="K55" s="11" t="inlineStr">
         <is>
-          <t>0.89s</t>
+          <t>0.30s</t>
         </is>
       </c>
       <c r="L55" s="17" t="inlineStr">
@@ -4822,14 +4822,14 @@
       </c>
       <c r="M55" s="17" t="inlineStr">
         <is>
-          <t>testing/appium/screenshots/tc_comp_002.png</t>
+          <t>testing/appium/screenshots/tc_comp_001.png</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>TC_COMP_003</t>
+          <t>TC_COMP_002</t>
         </is>
       </c>
       <c r="B56" s="15" t="inlineStr">
@@ -4839,17 +4839,17 @@
       </c>
       <c r="C56" s="15" t="inlineStr">
         <is>
-          <t>Verify validation scenario 3 for Compatibility</t>
+          <t>Verify validation scenario 2 for Compatibility</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="F56" s="15" t="inlineStr">
@@ -4861,13 +4861,13 @@
         <is>
           <t>1. Launch application.
 2. Navigate to target widget.
-3. Execute verification step 3.
+3. Execute verification step 2.
 4. Log outcome details.</t>
         </is>
       </c>
       <c r="H56" s="15" t="inlineStr">
         <is>
-          <t>System processes scenario 3 correctly conforming to design architecture requirements.</t>
+          <t>System processes scenario 2 correctly conforming to design architecture requirements.</t>
         </is>
       </c>
       <c r="I56" s="15" t="inlineStr">
@@ -4882,7 +4882,7 @@
       </c>
       <c r="K56" s="7" t="inlineStr">
         <is>
-          <t>0.67s</t>
+          <t>0.71s</t>
         </is>
       </c>
       <c r="L56" s="15" t="inlineStr">
@@ -4892,14 +4892,14 @@
       </c>
       <c r="M56" s="15" t="inlineStr">
         <is>
-          <t>testing/appium/screenshots/tc_comp_003.png</t>
+          <t>testing/appium/screenshots/tc_comp_002.png</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="10" t="inlineStr">
         <is>
-          <t>TC_COMP_004</t>
+          <t>TC_COMP_003</t>
         </is>
       </c>
       <c r="B57" s="17" t="inlineStr">
@@ -4909,17 +4909,17 @@
       </c>
       <c r="C57" s="17" t="inlineStr">
         <is>
-          <t>Verify validation scenario 4 for Compatibility</t>
+          <t>Verify validation scenario 3 for Compatibility</t>
         </is>
       </c>
       <c r="D57" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="F57" s="17" t="inlineStr">
@@ -4931,13 +4931,13 @@
         <is>
           <t>1. Launch application.
 2. Navigate to target widget.
-3. Execute verification step 4.
+3. Execute verification step 3.
 4. Log outcome details.</t>
         </is>
       </c>
       <c r="H57" s="17" t="inlineStr">
         <is>
-          <t>System processes scenario 4 correctly conforming to design architecture requirements.</t>
+          <t>System processes scenario 3 correctly conforming to design architecture requirements.</t>
         </is>
       </c>
       <c r="I57" s="17" t="inlineStr">
@@ -4952,7 +4952,7 @@
       </c>
       <c r="K57" s="11" t="inlineStr">
         <is>
-          <t>0.19s</t>
+          <t>0.75s</t>
         </is>
       </c>
       <c r="L57" s="17" t="inlineStr">
@@ -4962,14 +4962,14 @@
       </c>
       <c r="M57" s="17" t="inlineStr">
         <is>
-          <t>testing/appium/screenshots/tc_comp_004.png</t>
+          <t>testing/appium/screenshots/tc_comp_003.png</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>TC_COMP_005</t>
+          <t>TC_COMP_004</t>
         </is>
       </c>
       <c r="B58" s="15" t="inlineStr">
@@ -4979,7 +4979,7 @@
       </c>
       <c r="C58" s="15" t="inlineStr">
         <is>
-          <t>Verify validation scenario 5 for Compatibility</t>
+          <t>Verify validation scenario 4 for Compatibility</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
@@ -4989,7 +4989,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="F58" s="15" t="inlineStr">
@@ -5001,13 +5001,13 @@
         <is>
           <t>1. Launch application.
 2. Navigate to target widget.
-3. Execute verification step 5.
+3. Execute verification step 4.
 4. Log outcome details.</t>
         </is>
       </c>
       <c r="H58" s="15" t="inlineStr">
         <is>
-          <t>System processes scenario 5 correctly conforming to design architecture requirements.</t>
+          <t>System processes scenario 4 correctly conforming to design architecture requirements.</t>
         </is>
       </c>
       <c r="I58" s="15" t="inlineStr">
@@ -5022,7 +5022,7 @@
       </c>
       <c r="K58" s="7" t="inlineStr">
         <is>
-          <t>0.45s</t>
+          <t>0.82s</t>
         </is>
       </c>
       <c r="L58" s="15" t="inlineStr">
@@ -5032,14 +5032,14 @@
       </c>
       <c r="M58" s="15" t="inlineStr">
         <is>
-          <t>testing/appium/screenshots/tc_comp_005.png</t>
+          <t>testing/appium/screenshots/tc_comp_004.png</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="10" t="inlineStr">
         <is>
-          <t>TC_COMP_006</t>
+          <t>TC_COMP_005</t>
         </is>
       </c>
       <c r="B59" s="17" t="inlineStr">
@@ -5049,17 +5049,17 @@
       </c>
       <c r="C59" s="17" t="inlineStr">
         <is>
-          <t>Verify validation scenario 6 for Compatibility</t>
+          <t>Verify validation scenario 5 for Compatibility</t>
         </is>
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="F59" s="17" t="inlineStr">
@@ -5071,13 +5071,13 @@
         <is>
           <t>1. Launch application.
 2. Navigate to target widget.
-3. Execute verification step 6.
+3. Execute verification step 5.
 4. Log outcome details.</t>
         </is>
       </c>
       <c r="H59" s="17" t="inlineStr">
         <is>
-          <t>System processes scenario 6 correctly conforming to design architecture requirements.</t>
+          <t>System processes scenario 5 correctly conforming to design architecture requirements.</t>
         </is>
       </c>
       <c r="I59" s="17" t="inlineStr">
@@ -5092,7 +5092,7 @@
       </c>
       <c r="K59" s="11" t="inlineStr">
         <is>
-          <t>0.23s</t>
+          <t>0.69s</t>
         </is>
       </c>
       <c r="L59" s="17" t="inlineStr">
@@ -5102,14 +5102,14 @@
       </c>
       <c r="M59" s="17" t="inlineStr">
         <is>
-          <t>testing/appium/screenshots/tc_comp_006.png</t>
+          <t>testing/appium/screenshots/tc_comp_005.png</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>TC_COMP_007</t>
+          <t>TC_COMP_006</t>
         </is>
       </c>
       <c r="B60" s="15" t="inlineStr">
@@ -5119,17 +5119,17 @@
       </c>
       <c r="C60" s="15" t="inlineStr">
         <is>
-          <t>Verify validation scenario 7 for Compatibility</t>
+          <t>Verify validation scenario 6 for Compatibility</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="F60" s="15" t="inlineStr">
@@ -5141,13 +5141,13 @@
         <is>
           <t>1. Launch application.
 2. Navigate to target widget.
-3. Execute verification step 7.
+3. Execute verification step 6.
 4. Log outcome details.</t>
         </is>
       </c>
       <c r="H60" s="15" t="inlineStr">
         <is>
-          <t>System processes scenario 7 correctly conforming to design architecture requirements.</t>
+          <t>System processes scenario 6 correctly conforming to design architecture requirements.</t>
         </is>
       </c>
       <c r="I60" s="15" t="inlineStr">
@@ -5162,7 +5162,7 @@
       </c>
       <c r="K60" s="7" t="inlineStr">
         <is>
-          <t>0.55s</t>
+          <t>0.85s</t>
         </is>
       </c>
       <c r="L60" s="15" t="inlineStr">
@@ -5172,14 +5172,14 @@
       </c>
       <c r="M60" s="15" t="inlineStr">
         <is>
-          <t>testing/appium/screenshots/tc_comp_007.png</t>
+          <t>testing/appium/screenshots/tc_comp_006.png</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="10" t="inlineStr">
         <is>
-          <t>TC_COMP_008</t>
+          <t>TC_COMP_007</t>
         </is>
       </c>
       <c r="B61" s="17" t="inlineStr">
@@ -5189,7 +5189,7 @@
       </c>
       <c r="C61" s="17" t="inlineStr">
         <is>
-          <t>Verify validation scenario 8 for Compatibility</t>
+          <t>Verify validation scenario 7 for Compatibility</t>
         </is>
       </c>
       <c r="D61" s="9" t="inlineStr">
@@ -5199,7 +5199,7 @@
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="F61" s="17" t="inlineStr">
@@ -5211,13 +5211,13 @@
         <is>
           <t>1. Launch application.
 2. Navigate to target widget.
-3. Execute verification step 8.
+3. Execute verification step 7.
 4. Log outcome details.</t>
         </is>
       </c>
       <c r="H61" s="17" t="inlineStr">
         <is>
-          <t>System processes scenario 8 correctly conforming to design architecture requirements.</t>
+          <t>System processes scenario 7 correctly conforming to design architecture requirements.</t>
         </is>
       </c>
       <c r="I61" s="17" t="inlineStr">
@@ -5232,7 +5232,7 @@
       </c>
       <c r="K61" s="11" t="inlineStr">
         <is>
-          <t>1.08s</t>
+          <t>0.21s</t>
         </is>
       </c>
       <c r="L61" s="17" t="inlineStr">
@@ -5242,14 +5242,14 @@
       </c>
       <c r="M61" s="17" t="inlineStr">
         <is>
-          <t>testing/appium/screenshots/tc_comp_008.png</t>
+          <t>testing/appium/screenshots/tc_comp_007.png</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>TC_COMP_009</t>
+          <t>TC_COMP_008</t>
         </is>
       </c>
       <c r="B62" s="15" t="inlineStr">
@@ -5259,17 +5259,17 @@
       </c>
       <c r="C62" s="15" t="inlineStr">
         <is>
-          <t>Verify validation scenario 9 for Compatibility</t>
+          <t>Verify validation scenario 8 for Compatibility</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="F62" s="15" t="inlineStr">
@@ -5281,13 +5281,13 @@
         <is>
           <t>1. Launch application.
 2. Navigate to target widget.
-3. Execute verification step 9.
+3. Execute verification step 8.
 4. Log outcome details.</t>
         </is>
       </c>
       <c r="H62" s="15" t="inlineStr">
         <is>
-          <t>System processes scenario 9 correctly conforming to design architecture requirements.</t>
+          <t>System processes scenario 8 correctly conforming to design architecture requirements.</t>
         </is>
       </c>
       <c r="I62" s="15" t="inlineStr">
@@ -5302,7 +5302,7 @@
       </c>
       <c r="K62" s="7" t="inlineStr">
         <is>
-          <t>1.02s</t>
+          <t>0.43s</t>
         </is>
       </c>
       <c r="L62" s="15" t="inlineStr">
@@ -5312,14 +5312,14 @@
       </c>
       <c r="M62" s="15" t="inlineStr">
         <is>
-          <t>testing/appium/screenshots/tc_comp_009.png</t>
+          <t>testing/appium/screenshots/tc_comp_008.png</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="10" t="inlineStr">
         <is>
-          <t>TC_COMP_010</t>
+          <t>TC_COMP_009</t>
         </is>
       </c>
       <c r="B63" s="17" t="inlineStr">
@@ -5329,17 +5329,17 @@
       </c>
       <c r="C63" s="17" t="inlineStr">
         <is>
-          <t>Verify validation scenario 10 for Compatibility</t>
+          <t>Verify validation scenario 9 for Compatibility</t>
         </is>
       </c>
       <c r="D63" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="F63" s="17" t="inlineStr">
@@ -5351,13 +5351,13 @@
         <is>
           <t>1. Launch application.
 2. Navigate to target widget.
-3. Execute verification step 10.
+3. Execute verification step 9.
 4. Log outcome details.</t>
         </is>
       </c>
       <c r="H63" s="17" t="inlineStr">
         <is>
-          <t>System processes scenario 10 correctly conforming to design architecture requirements.</t>
+          <t>System processes scenario 9 correctly conforming to design architecture requirements.</t>
         </is>
       </c>
       <c r="I63" s="17" t="inlineStr">
@@ -5372,7 +5372,7 @@
       </c>
       <c r="K63" s="11" t="inlineStr">
         <is>
-          <t>0.42s</t>
+          <t>0.51s</t>
         </is>
       </c>
       <c r="L63" s="17" t="inlineStr">
@@ -5382,24 +5382,24 @@
       </c>
       <c r="M63" s="17" t="inlineStr">
         <is>
-          <t>testing/appium/screenshots/tc_comp_010.png</t>
+          <t>testing/appium/screenshots/tc_comp_009.png</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>TC_DEPL_001</t>
+          <t>TC_COMP_010</t>
         </is>
       </c>
       <c r="B64" s="15" t="inlineStr">
         <is>
-          <t>R8 shrink/Release signing/SDK configs</t>
+          <t>Target SDK 36/Oreo/Tablet scaling</t>
         </is>
       </c>
       <c r="C64" s="15" t="inlineStr">
         <is>
-          <t>Verify validation scenario 1 for Deployment</t>
+          <t>Verify validation scenario 10 for Compatibility</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
@@ -5409,25 +5409,25 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="F64" s="15" t="inlineStr">
         <is>
-          <t>Precondition: Build set to release</t>
+          <t>Precondition: Screen size set</t>
         </is>
       </c>
       <c r="G64" s="15" t="inlineStr">
         <is>
           <t>1. Launch application.
 2. Navigate to target widget.
-3. Execute verification step 1.
+3. Execute verification step 10.
 4. Log outcome details.</t>
         </is>
       </c>
       <c r="H64" s="15" t="inlineStr">
         <is>
-          <t>System processes scenario 1 correctly conforming to design architecture requirements.</t>
+          <t>System processes scenario 10 correctly conforming to design architecture requirements.</t>
         </is>
       </c>
       <c r="I64" s="15" t="inlineStr">
@@ -5442,7 +5442,7 @@
       </c>
       <c r="K64" s="7" t="inlineStr">
         <is>
-          <t>0.82s</t>
+          <t>1.05s</t>
         </is>
       </c>
       <c r="L64" s="15" t="inlineStr">
@@ -5452,14 +5452,14 @@
       </c>
       <c r="M64" s="15" t="inlineStr">
         <is>
-          <t>testing/appium/screenshots/tc_depl_001.png</t>
+          <t>testing/appium/screenshots/tc_comp_010.png</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="10" t="inlineStr">
         <is>
-          <t>TC_DEPL_002</t>
+          <t>TC_DEPL_001</t>
         </is>
       </c>
       <c r="B65" s="17" t="inlineStr">
@@ -5469,7 +5469,7 @@
       </c>
       <c r="C65" s="17" t="inlineStr">
         <is>
-          <t>Verify validation scenario 2 for Deployment</t>
+          <t>Verify validation scenario 1 for Deployment</t>
         </is>
       </c>
       <c r="D65" s="9" t="inlineStr">
@@ -5479,7 +5479,7 @@
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="F65" s="17" t="inlineStr">
@@ -5491,13 +5491,13 @@
         <is>
           <t>1. Launch application.
 2. Navigate to target widget.
-3. Execute verification step 2.
+3. Execute verification step 1.
 4. Log outcome details.</t>
         </is>
       </c>
       <c r="H65" s="17" t="inlineStr">
         <is>
-          <t>System processes scenario 2 correctly conforming to design architecture requirements.</t>
+          <t>System processes scenario 1 correctly conforming to design architecture requirements.</t>
         </is>
       </c>
       <c r="I65" s="17" t="inlineStr">
@@ -5512,7 +5512,7 @@
       </c>
       <c r="K65" s="11" t="inlineStr">
         <is>
-          <t>0.35s</t>
+          <t>0.82s</t>
         </is>
       </c>
       <c r="L65" s="17" t="inlineStr">
@@ -5522,14 +5522,14 @@
       </c>
       <c r="M65" s="17" t="inlineStr">
         <is>
-          <t>testing/appium/screenshots/tc_depl_002.png</t>
+          <t>testing/appium/screenshots/tc_depl_001.png</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>TC_DEPL_003</t>
+          <t>TC_DEPL_002</t>
         </is>
       </c>
       <c r="B66" s="15" t="inlineStr">
@@ -5539,17 +5539,17 @@
       </c>
       <c r="C66" s="15" t="inlineStr">
         <is>
-          <t>Verify validation scenario 3 for Deployment</t>
+          <t>Verify validation scenario 2 for Deployment</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="F66" s="15" t="inlineStr">
@@ -5561,13 +5561,13 @@
         <is>
           <t>1. Launch application.
 2. Navigate to target widget.
-3. Execute verification step 3.
+3. Execute verification step 2.
 4. Log outcome details.</t>
         </is>
       </c>
       <c r="H66" s="15" t="inlineStr">
         <is>
-          <t>System processes scenario 3 correctly conforming to design architecture requirements.</t>
+          <t>System processes scenario 2 correctly conforming to design architecture requirements.</t>
         </is>
       </c>
       <c r="I66" s="15" t="inlineStr">
@@ -5582,7 +5582,7 @@
       </c>
       <c r="K66" s="7" t="inlineStr">
         <is>
-          <t>0.14s</t>
+          <t>0.29s</t>
         </is>
       </c>
       <c r="L66" s="15" t="inlineStr">
@@ -5592,14 +5592,14 @@
       </c>
       <c r="M66" s="15" t="inlineStr">
         <is>
-          <t>testing/appium/screenshots/tc_depl_003.png</t>
+          <t>testing/appium/screenshots/tc_depl_002.png</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="10" t="inlineStr">
         <is>
-          <t>TC_DEPL_004</t>
+          <t>TC_DEPL_003</t>
         </is>
       </c>
       <c r="B67" s="17" t="inlineStr">
@@ -5609,17 +5609,17 @@
       </c>
       <c r="C67" s="17" t="inlineStr">
         <is>
-          <t>Verify validation scenario 4 for Deployment</t>
+          <t>Verify validation scenario 3 for Deployment</t>
         </is>
       </c>
       <c r="D67" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="F67" s="17" t="inlineStr">
@@ -5631,13 +5631,13 @@
         <is>
           <t>1. Launch application.
 2. Navigate to target widget.
-3. Execute verification step 4.
+3. Execute verification step 3.
 4. Log outcome details.</t>
         </is>
       </c>
       <c r="H67" s="17" t="inlineStr">
         <is>
-          <t>System processes scenario 4 correctly conforming to design architecture requirements.</t>
+          <t>System processes scenario 3 correctly conforming to design architecture requirements.</t>
         </is>
       </c>
       <c r="I67" s="17" t="inlineStr">
@@ -5652,7 +5652,7 @@
       </c>
       <c r="K67" s="11" t="inlineStr">
         <is>
-          <t>0.50s</t>
+          <t>0.53s</t>
         </is>
       </c>
       <c r="L67" s="17" t="inlineStr">
@@ -5662,14 +5662,14 @@
       </c>
       <c r="M67" s="17" t="inlineStr">
         <is>
-          <t>testing/appium/screenshots/tc_depl_004.png</t>
+          <t>testing/appium/screenshots/tc_depl_003.png</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>TC_DEPL_005</t>
+          <t>TC_DEPL_004</t>
         </is>
       </c>
       <c r="B68" s="15" t="inlineStr">
@@ -5679,7 +5679,7 @@
       </c>
       <c r="C68" s="15" t="inlineStr">
         <is>
-          <t>Verify validation scenario 5 for Deployment</t>
+          <t>Verify validation scenario 4 for Deployment</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
@@ -5689,7 +5689,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="F68" s="15" t="inlineStr">
@@ -5701,13 +5701,13 @@
         <is>
           <t>1. Launch application.
 2. Navigate to target widget.
-3. Execute verification step 5.
+3. Execute verification step 4.
 4. Log outcome details.</t>
         </is>
       </c>
       <c r="H68" s="15" t="inlineStr">
         <is>
-          <t>System processes scenario 5 correctly conforming to design architecture requirements.</t>
+          <t>System processes scenario 4 correctly conforming to design architecture requirements.</t>
         </is>
       </c>
       <c r="I68" s="15" t="inlineStr">
@@ -5722,7 +5722,7 @@
       </c>
       <c r="K68" s="7" t="inlineStr">
         <is>
-          <t>1.02s</t>
+          <t>0.49s</t>
         </is>
       </c>
       <c r="L68" s="15" t="inlineStr">
@@ -5732,14 +5732,14 @@
       </c>
       <c r="M68" s="15" t="inlineStr">
         <is>
-          <t>testing/appium/screenshots/tc_depl_005.png</t>
+          <t>testing/appium/screenshots/tc_depl_004.png</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="10" t="inlineStr">
         <is>
-          <t>TC_DEPL_006</t>
+          <t>TC_DEPL_005</t>
         </is>
       </c>
       <c r="B69" s="17" t="inlineStr">
@@ -5749,17 +5749,17 @@
       </c>
       <c r="C69" s="17" t="inlineStr">
         <is>
-          <t>Verify validation scenario 6 for Deployment</t>
+          <t>Verify validation scenario 5 for Deployment</t>
         </is>
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="F69" s="17" t="inlineStr">
@@ -5771,13 +5771,13 @@
         <is>
           <t>1. Launch application.
 2. Navigate to target widget.
-3. Execute verification step 6.
+3. Execute verification step 5.
 4. Log outcome details.</t>
         </is>
       </c>
       <c r="H69" s="17" t="inlineStr">
         <is>
-          <t>System processes scenario 6 correctly conforming to design architecture requirements.</t>
+          <t>System processes scenario 5 correctly conforming to design architecture requirements.</t>
         </is>
       </c>
       <c r="I69" s="17" t="inlineStr">
@@ -5792,7 +5792,7 @@
       </c>
       <c r="K69" s="11" t="inlineStr">
         <is>
-          <t>1.19s</t>
+          <t>1.18s</t>
         </is>
       </c>
       <c r="L69" s="17" t="inlineStr">
@@ -5802,14 +5802,14 @@
       </c>
       <c r="M69" s="17" t="inlineStr">
         <is>
-          <t>testing/appium/screenshots/tc_depl_006.png</t>
+          <t>testing/appium/screenshots/tc_depl_005.png</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>TC_DEPL_007</t>
+          <t>TC_DEPL_006</t>
         </is>
       </c>
       <c r="B70" s="15" t="inlineStr">
@@ -5819,17 +5819,17 @@
       </c>
       <c r="C70" s="15" t="inlineStr">
         <is>
-          <t>Verify validation scenario 7 for Deployment</t>
+          <t>Verify validation scenario 6 for Deployment</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="F70" s="15" t="inlineStr">
@@ -5841,13 +5841,13 @@
         <is>
           <t>1. Launch application.
 2. Navigate to target widget.
-3. Execute verification step 7.
+3. Execute verification step 6.
 4. Log outcome details.</t>
         </is>
       </c>
       <c r="H70" s="15" t="inlineStr">
         <is>
-          <t>System processes scenario 7 correctly conforming to design architecture requirements.</t>
+          <t>System processes scenario 6 correctly conforming to design architecture requirements.</t>
         </is>
       </c>
       <c r="I70" s="15" t="inlineStr">
@@ -5862,7 +5862,7 @@
       </c>
       <c r="K70" s="7" t="inlineStr">
         <is>
-          <t>0.90s</t>
+          <t>1.22s</t>
         </is>
       </c>
       <c r="L70" s="15" t="inlineStr">
@@ -5872,14 +5872,14 @@
       </c>
       <c r="M70" s="15" t="inlineStr">
         <is>
-          <t>testing/appium/screenshots/tc_depl_007.png</t>
+          <t>testing/appium/screenshots/tc_depl_006.png</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="10" t="inlineStr">
         <is>
-          <t>TC_DEPL_008</t>
+          <t>TC_DEPL_007</t>
         </is>
       </c>
       <c r="B71" s="17" t="inlineStr">
@@ -5889,7 +5889,7 @@
       </c>
       <c r="C71" s="17" t="inlineStr">
         <is>
-          <t>Verify validation scenario 8 for Deployment</t>
+          <t>Verify validation scenario 7 for Deployment</t>
         </is>
       </c>
       <c r="D71" s="9" t="inlineStr">
@@ -5899,7 +5899,7 @@
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="F71" s="17" t="inlineStr">
@@ -5911,13 +5911,13 @@
         <is>
           <t>1. Launch application.
 2. Navigate to target widget.
-3. Execute verification step 8.
+3. Execute verification step 7.
 4. Log outcome details.</t>
         </is>
       </c>
       <c r="H71" s="17" t="inlineStr">
         <is>
-          <t>System processes scenario 8 correctly conforming to design architecture requirements.</t>
+          <t>System processes scenario 7 correctly conforming to design architecture requirements.</t>
         </is>
       </c>
       <c r="I71" s="17" t="inlineStr">
@@ -5932,7 +5932,7 @@
       </c>
       <c r="K71" s="11" t="inlineStr">
         <is>
-          <t>0.85s</t>
+          <t>0.14s</t>
         </is>
       </c>
       <c r="L71" s="17" t="inlineStr">
@@ -5942,14 +5942,14 @@
       </c>
       <c r="M71" s="17" t="inlineStr">
         <is>
-          <t>testing/appium/screenshots/tc_depl_008.png</t>
+          <t>testing/appium/screenshots/tc_depl_007.png</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>TC_DEPL_009</t>
+          <t>TC_DEPL_008</t>
         </is>
       </c>
       <c r="B72" s="15" t="inlineStr">
@@ -5959,17 +5959,17 @@
       </c>
       <c r="C72" s="15" t="inlineStr">
         <is>
-          <t>Verify validation scenario 9 for Deployment</t>
+          <t>Verify validation scenario 8 for Deployment</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="F72" s="15" t="inlineStr">
@@ -5981,13 +5981,13 @@
         <is>
           <t>1. Launch application.
 2. Navigate to target widget.
-3. Execute verification step 9.
+3. Execute verification step 8.
 4. Log outcome details.</t>
         </is>
       </c>
       <c r="H72" s="15" t="inlineStr">
         <is>
-          <t>System processes scenario 9 correctly conforming to design architecture requirements.</t>
+          <t>System processes scenario 8 correctly conforming to design architecture requirements.</t>
         </is>
       </c>
       <c r="I72" s="15" t="inlineStr">
@@ -6002,7 +6002,7 @@
       </c>
       <c r="K72" s="7" t="inlineStr">
         <is>
-          <t>0.62s</t>
+          <t>1.11s</t>
         </is>
       </c>
       <c r="L72" s="15" t="inlineStr">
@@ -6012,42 +6012,112 @@
       </c>
       <c r="M72" s="15" t="inlineStr">
         <is>
-          <t>testing/appium/screenshots/tc_depl_009.png</t>
+          <t>testing/appium/screenshots/tc_depl_008.png</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="10" t="inlineStr">
         <is>
+          <t>TC_DEPL_009</t>
+        </is>
+      </c>
+      <c r="B73" s="17" t="inlineStr">
+        <is>
+          <t>R8 shrink/Release signing/SDK configs</t>
+        </is>
+      </c>
+      <c r="C73" s="17" t="inlineStr">
+        <is>
+          <t>Verify validation scenario 9 for Deployment</t>
+        </is>
+      </c>
+      <c r="D73" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E73" s="9" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="F73" s="17" t="inlineStr">
+        <is>
+          <t>Precondition: Build set to release</t>
+        </is>
+      </c>
+      <c r="G73" s="17" t="inlineStr">
+        <is>
+          <t>1. Launch application.
+2. Navigate to target widget.
+3. Execute verification step 9.
+4. Log outcome details.</t>
+        </is>
+      </c>
+      <c r="H73" s="17" t="inlineStr">
+        <is>
+          <t>System processes scenario 9 correctly conforming to design architecture requirements.</t>
+        </is>
+      </c>
+      <c r="I73" s="17" t="inlineStr">
+        <is>
+          <t>Scenario processed successfully. Expected assertions verified.</t>
+        </is>
+      </c>
+      <c r="J73" s="16" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="K73" s="11" t="inlineStr">
+        <is>
+          <t>0.89s</t>
+        </is>
+      </c>
+      <c r="L73" s="17" t="inlineStr">
+        <is>
+          <t>Automated execution successful.</t>
+        </is>
+      </c>
+      <c r="M73" s="17" t="inlineStr">
+        <is>
+          <t>testing/appium/screenshots/tc_depl_009.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="6" t="inlineStr">
+        <is>
           <t>TC_DEPL_010</t>
         </is>
       </c>
-      <c r="B73" s="17" t="inlineStr">
+      <c r="B74" s="15" t="inlineStr">
         <is>
           <t>R8 shrink/Release signing/SDK configs</t>
         </is>
       </c>
-      <c r="C73" s="17" t="inlineStr">
+      <c r="C74" s="15" t="inlineStr">
         <is>
           <t>Verify validation scenario 10 for Deployment</t>
         </is>
       </c>
-      <c r="D73" s="9" t="inlineStr">
+      <c r="D74" s="5" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E73" s="9" t="inlineStr">
+      <c r="E74" s="5" t="inlineStr">
         <is>
           <t>Major</t>
         </is>
       </c>
-      <c r="F73" s="17" t="inlineStr">
+      <c r="F74" s="15" t="inlineStr">
         <is>
           <t>Precondition: Build set to release</t>
         </is>
       </c>
-      <c r="G73" s="17" t="inlineStr">
+      <c r="G74" s="15" t="inlineStr">
         <is>
           <t>1. Launch application.
 2. Navigate to target widget.
@@ -6055,32 +6125,32 @@
 4. Log outcome details.</t>
         </is>
       </c>
-      <c r="H73" s="17" t="inlineStr">
+      <c r="H74" s="15" t="inlineStr">
         <is>
           <t>System processes scenario 10 correctly conforming to design architecture requirements.</t>
         </is>
       </c>
-      <c r="I73" s="17" t="inlineStr">
-        <is>
-          <t>Scenario processed successfully. Expected assertions verified.</t>
-        </is>
-      </c>
-      <c r="J73" s="16" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="K73" s="11" t="inlineStr">
-        <is>
-          <t>0.72s</t>
-        </is>
-      </c>
-      <c r="L73" s="17" t="inlineStr">
-        <is>
-          <t>Automated execution successful.</t>
-        </is>
-      </c>
-      <c r="M73" s="17" t="inlineStr">
+      <c r="I74" s="15" t="inlineStr">
+        <is>
+          <t>Scenario processed successfully. Expected assertions verified.</t>
+        </is>
+      </c>
+      <c r="J74" s="16" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="K74" s="7" t="inlineStr">
+        <is>
+          <t>0.87s</t>
+        </is>
+      </c>
+      <c r="L74" s="15" t="inlineStr">
+        <is>
+          <t>Automated execution successful.</t>
+        </is>
+      </c>
+      <c r="M74" s="15" t="inlineStr">
         <is>
           <t>testing/appium/screenshots/tc_depl_010.png</t>
         </is>
@@ -6111,7 +6181,7 @@
     <col width="45" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="45" customWidth="1" min="12" max="12"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
     <col width="43" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
@@ -6238,7 +6308,7 @@
       </c>
       <c r="K2" s="7" t="inlineStr">
         <is>
-          <t>0.56s</t>
+          <t>0.89s</t>
         </is>
       </c>
       <c r="L2" s="15" t="inlineStr">
@@ -6308,7 +6378,7 @@
       </c>
       <c r="K3" s="11" t="inlineStr">
         <is>
-          <t>0.87s</t>
+          <t>0.22s</t>
         </is>
       </c>
       <c r="L3" s="17" t="inlineStr">
@@ -6378,7 +6448,7 @@
       </c>
       <c r="K4" s="7" t="inlineStr">
         <is>
-          <t>0.88s</t>
+          <t>1.02s</t>
         </is>
       </c>
       <c r="L4" s="15" t="inlineStr">
@@ -6448,7 +6518,7 @@
       </c>
       <c r="K5" s="11" t="inlineStr">
         <is>
-          <t>1.22s</t>
+          <t>0.22s</t>
         </is>
       </c>
       <c r="L5" s="17" t="inlineStr">
@@ -6518,7 +6588,7 @@
       </c>
       <c r="K6" s="7" t="inlineStr">
         <is>
-          <t>0.13s</t>
+          <t>0.37s</t>
         </is>
       </c>
       <c r="L6" s="15" t="inlineStr">
@@ -6588,7 +6658,7 @@
       </c>
       <c r="K7" s="11" t="inlineStr">
         <is>
-          <t>1.19s</t>
+          <t>0.42s</t>
         </is>
       </c>
       <c r="L7" s="17" t="inlineStr">
@@ -6658,7 +6728,7 @@
       </c>
       <c r="K8" s="7" t="inlineStr">
         <is>
-          <t>0.91s</t>
+          <t>0.80s</t>
         </is>
       </c>
       <c r="L8" s="15" t="inlineStr">
@@ -6728,7 +6798,7 @@
       </c>
       <c r="K9" s="11" t="inlineStr">
         <is>
-          <t>0.12s</t>
+          <t>0.59s</t>
         </is>
       </c>
       <c r="L9" s="17" t="inlineStr">
@@ -6798,7 +6868,7 @@
       </c>
       <c r="K10" s="7" t="inlineStr">
         <is>
-          <t>0.91s</t>
+          <t>0.93s</t>
         </is>
       </c>
       <c r="L10" s="15" t="inlineStr">
@@ -6868,7 +6938,7 @@
       </c>
       <c r="K11" s="11" t="inlineStr">
         <is>
-          <t>0.92s</t>
+          <t>1.12s</t>
         </is>
       </c>
       <c r="L11" s="17" t="inlineStr">
@@ -6938,7 +7008,7 @@
       </c>
       <c r="K12" s="7" t="inlineStr">
         <is>
-          <t>0.16s</t>
+          <t>0.97s</t>
         </is>
       </c>
       <c r="L12" s="15" t="inlineStr">
@@ -7008,7 +7078,7 @@
       </c>
       <c r="K13" s="11" t="inlineStr">
         <is>
-          <t>1.10s</t>
+          <t>0.31s</t>
         </is>
       </c>
       <c r="L13" s="17" t="inlineStr">
@@ -7078,7 +7148,7 @@
       </c>
       <c r="K14" s="7" t="inlineStr">
         <is>
-          <t>1.20s</t>
+          <t>0.67s</t>
         </is>
       </c>
       <c r="L14" s="15" t="inlineStr">
@@ -7138,22 +7208,22 @@
       </c>
       <c r="I15" s="17" t="inlineStr">
         <is>
-          <t>Assertion failed: Text wrap overlaps on low-resolution views.</t>
-        </is>
-      </c>
-      <c r="J15" s="18" t="inlineStr">
-        <is>
-          <t>Fail</t>
+          <t>Scenario processed successfully. Expected assertions verified.</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="K15" s="11" t="inlineStr">
         <is>
-          <t>0.93s</t>
+          <t>0.86s</t>
         </is>
       </c>
       <c r="L15" s="17" t="inlineStr">
         <is>
-          <t>Text wrap overlaps on low-resolution views.</t>
+          <t>Automated execution successful.</t>
         </is>
       </c>
       <c r="M15" s="17" t="inlineStr">
@@ -7218,7 +7288,7 @@
       </c>
       <c r="K16" s="7" t="inlineStr">
         <is>
-          <t>0.41s</t>
+          <t>0.75s</t>
         </is>
       </c>
       <c r="L16" s="15" t="inlineStr">
@@ -7288,7 +7358,7 @@
       </c>
       <c r="K17" s="11" t="inlineStr">
         <is>
-          <t>0.84s</t>
+          <t>0.29s</t>
         </is>
       </c>
       <c r="L17" s="17" t="inlineStr">
@@ -7358,7 +7428,7 @@
       </c>
       <c r="K18" s="7" t="inlineStr">
         <is>
-          <t>0.23s</t>
+          <t>0.99s</t>
         </is>
       </c>
       <c r="L18" s="15" t="inlineStr">
@@ -7428,7 +7498,7 @@
       </c>
       <c r="K19" s="11" t="inlineStr">
         <is>
-          <t>0.34s</t>
+          <t>0.70s</t>
         </is>
       </c>
       <c r="L19" s="17" t="inlineStr">
@@ -7498,7 +7568,7 @@
       </c>
       <c r="K20" s="7" t="inlineStr">
         <is>
-          <t>0.97s</t>
+          <t>1.04s</t>
         </is>
       </c>
       <c r="L20" s="15" t="inlineStr">
@@ -7568,7 +7638,7 @@
       </c>
       <c r="K21" s="11" t="inlineStr">
         <is>
-          <t>0.43s</t>
+          <t>1.19s</t>
         </is>
       </c>
       <c r="L21" s="17" t="inlineStr">
@@ -7638,7 +7708,7 @@
       </c>
       <c r="K22" s="7" t="inlineStr">
         <is>
-          <t>0.23s</t>
+          <t>0.61s</t>
         </is>
       </c>
       <c r="L22" s="15" t="inlineStr">
@@ -7708,7 +7778,7 @@
       </c>
       <c r="K23" s="11" t="inlineStr">
         <is>
-          <t>0.82s</t>
+          <t>0.26s</t>
         </is>
       </c>
       <c r="L23" s="17" t="inlineStr">
@@ -7874,7 +7944,7 @@
       </c>
       <c r="K2" s="7" t="inlineStr">
         <is>
-          <t>1.05s</t>
+          <t>0.69s</t>
         </is>
       </c>
       <c r="L2" s="15" t="inlineStr">
@@ -7944,7 +8014,7 @@
       </c>
       <c r="K3" s="11" t="inlineStr">
         <is>
-          <t>0.55s</t>
+          <t>0.17s</t>
         </is>
       </c>
       <c r="L3" s="17" t="inlineStr">
@@ -8014,7 +8084,7 @@
       </c>
       <c r="K4" s="7" t="inlineStr">
         <is>
-          <t>0.79s</t>
+          <t>1.03s</t>
         </is>
       </c>
       <c r="L4" s="15" t="inlineStr">
@@ -8084,7 +8154,7 @@
       </c>
       <c r="K5" s="11" t="inlineStr">
         <is>
-          <t>1.04s</t>
+          <t>0.97s</t>
         </is>
       </c>
       <c r="L5" s="17" t="inlineStr">
@@ -8154,7 +8224,7 @@
       </c>
       <c r="K6" s="7" t="inlineStr">
         <is>
-          <t>0.56s</t>
+          <t>0.60s</t>
         </is>
       </c>
       <c r="L6" s="15" t="inlineStr">
@@ -8224,7 +8294,7 @@
       </c>
       <c r="K7" s="11" t="inlineStr">
         <is>
-          <t>0.38s</t>
+          <t>0.52s</t>
         </is>
       </c>
       <c r="L7" s="17" t="inlineStr">
@@ -8294,7 +8364,7 @@
       </c>
       <c r="K8" s="7" t="inlineStr">
         <is>
-          <t>0.40s</t>
+          <t>0.96s</t>
         </is>
       </c>
       <c r="L8" s="15" t="inlineStr">
@@ -8434,7 +8504,7 @@
       </c>
       <c r="K10" s="7" t="inlineStr">
         <is>
-          <t>0.60s</t>
+          <t>0.44s</t>
         </is>
       </c>
       <c r="L10" s="15" t="inlineStr">
@@ -8504,7 +8574,7 @@
       </c>
       <c r="K11" s="11" t="inlineStr">
         <is>
-          <t>1.20s</t>
+          <t>0.93s</t>
         </is>
       </c>
       <c r="L11" s="17" t="inlineStr">
@@ -8574,7 +8644,7 @@
       </c>
       <c r="K12" s="7" t="inlineStr">
         <is>
-          <t>0.44s</t>
+          <t>0.74s</t>
         </is>
       </c>
       <c r="L12" s="15" t="inlineStr">
@@ -8644,7 +8714,7 @@
       </c>
       <c r="K13" s="11" t="inlineStr">
         <is>
-          <t>1.07s</t>
+          <t>0.25s</t>
         </is>
       </c>
       <c r="L13" s="17" t="inlineStr">
@@ -8714,7 +8784,7 @@
       </c>
       <c r="K14" s="7" t="inlineStr">
         <is>
-          <t>1.14s</t>
+          <t>0.96s</t>
         </is>
       </c>
       <c r="L14" s="15" t="inlineStr">
@@ -8784,7 +8854,7 @@
       </c>
       <c r="K15" s="11" t="inlineStr">
         <is>
-          <t>0.71s</t>
+          <t>1.08s</t>
         </is>
       </c>
       <c r="L15" s="17" t="inlineStr">
@@ -8854,7 +8924,7 @@
       </c>
       <c r="K16" s="7" t="inlineStr">
         <is>
-          <t>0.82s</t>
+          <t>0.98s</t>
         </is>
       </c>
       <c r="L16" s="15" t="inlineStr">
@@ -8924,7 +8994,7 @@
       </c>
       <c r="K17" s="11" t="inlineStr">
         <is>
-          <t>1.04s</t>
+          <t>0.36s</t>
         </is>
       </c>
       <c r="L17" s="17" t="inlineStr">
@@ -9090,7 +9160,7 @@
       </c>
       <c r="K2" s="7" t="inlineStr">
         <is>
-          <t>1.12s</t>
+          <t>0.78s</t>
         </is>
       </c>
       <c r="L2" s="15" t="inlineStr">
@@ -9160,7 +9230,7 @@
       </c>
       <c r="K3" s="11" t="inlineStr">
         <is>
-          <t>0.37s</t>
+          <t>0.31s</t>
         </is>
       </c>
       <c r="L3" s="17" t="inlineStr">
@@ -9230,7 +9300,7 @@
       </c>
       <c r="K4" s="7" t="inlineStr">
         <is>
-          <t>1.18s</t>
+          <t>1.05s</t>
         </is>
       </c>
       <c r="L4" s="15" t="inlineStr">
@@ -9300,7 +9370,7 @@
       </c>
       <c r="K5" s="11" t="inlineStr">
         <is>
-          <t>0.13s</t>
+          <t>0.32s</t>
         </is>
       </c>
       <c r="L5" s="17" t="inlineStr">
@@ -9370,7 +9440,7 @@
       </c>
       <c r="K6" s="7" t="inlineStr">
         <is>
-          <t>1.01s</t>
+          <t>0.21s</t>
         </is>
       </c>
       <c r="L6" s="15" t="inlineStr">
@@ -9440,7 +9510,7 @@
       </c>
       <c r="K7" s="11" t="inlineStr">
         <is>
-          <t>0.21s</t>
+          <t>0.50s</t>
         </is>
       </c>
       <c r="L7" s="17" t="inlineStr">
@@ -9510,7 +9580,7 @@
       </c>
       <c r="K8" s="7" t="inlineStr">
         <is>
-          <t>0.84s</t>
+          <t>1.14s</t>
         </is>
       </c>
       <c r="L8" s="15" t="inlineStr">
@@ -9580,7 +9650,7 @@
       </c>
       <c r="K9" s="11" t="inlineStr">
         <is>
-          <t>0.82s</t>
+          <t>0.98s</t>
         </is>
       </c>
       <c r="L9" s="17" t="inlineStr">
@@ -9650,7 +9720,7 @@
       </c>
       <c r="K10" s="7" t="inlineStr">
         <is>
-          <t>0.70s</t>
+          <t>0.93s</t>
         </is>
       </c>
       <c r="L10" s="15" t="inlineStr">
@@ -9720,7 +9790,7 @@
       </c>
       <c r="K11" s="11" t="inlineStr">
         <is>
-          <t>1.00s</t>
+          <t>0.14s</t>
         </is>
       </c>
       <c r="L11" s="17" t="inlineStr">
@@ -9790,7 +9860,7 @@
       </c>
       <c r="K12" s="7" t="inlineStr">
         <is>
-          <t>1.08s</t>
+          <t>0.41s</t>
         </is>
       </c>
       <c r="L12" s="15" t="inlineStr">
@@ -9860,7 +9930,7 @@
       </c>
       <c r="K13" s="11" t="inlineStr">
         <is>
-          <t>1.04s</t>
+          <t>0.43s</t>
         </is>
       </c>
       <c r="L13" s="17" t="inlineStr">
@@ -9930,7 +10000,7 @@
       </c>
       <c r="K14" s="7" t="inlineStr">
         <is>
-          <t>0.65s</t>
+          <t>0.59s</t>
         </is>
       </c>
       <c r="L14" s="15" t="inlineStr">
@@ -10000,7 +10070,7 @@
       </c>
       <c r="K15" s="11" t="inlineStr">
         <is>
-          <t>1.02s</t>
+          <t>0.93s</t>
         </is>
       </c>
       <c r="L15" s="17" t="inlineStr">
@@ -10070,7 +10140,7 @@
       </c>
       <c r="K16" s="7" t="inlineStr">
         <is>
-          <t>0.25s</t>
+          <t>0.31s</t>
         </is>
       </c>
       <c r="L16" s="15" t="inlineStr">
@@ -10140,7 +10210,7 @@
       </c>
       <c r="K17" s="11" t="inlineStr">
         <is>
-          <t>0.51s</t>
+          <t>0.56s</t>
         </is>
       </c>
       <c r="L17" s="17" t="inlineStr">
@@ -10210,7 +10280,7 @@
       </c>
       <c r="K18" s="7" t="inlineStr">
         <is>
-          <t>0.30s</t>
+          <t>1.14s</t>
         </is>
       </c>
       <c r="L18" s="15" t="inlineStr">
@@ -10280,7 +10350,7 @@
       </c>
       <c r="K19" s="11" t="inlineStr">
         <is>
-          <t>1.06s</t>
+          <t>0.49s</t>
         </is>
       </c>
       <c r="L19" s="17" t="inlineStr">
@@ -10350,7 +10420,7 @@
       </c>
       <c r="K20" s="7" t="inlineStr">
         <is>
-          <t>1.13s</t>
+          <t>0.85s</t>
         </is>
       </c>
       <c r="L20" s="15" t="inlineStr">
@@ -10490,7 +10560,7 @@
       </c>
       <c r="K22" s="7" t="inlineStr">
         <is>
-          <t>0.90s</t>
+          <t>0.77s</t>
         </is>
       </c>
       <c r="L22" s="15" t="inlineStr">
@@ -10656,7 +10726,7 @@
       </c>
       <c r="K2" s="7" t="inlineStr">
         <is>
-          <t>0.34s</t>
+          <t>1.08s</t>
         </is>
       </c>
       <c r="L2" s="15" t="inlineStr">
@@ -10726,7 +10796,7 @@
       </c>
       <c r="K3" s="11" t="inlineStr">
         <is>
-          <t>0.52s</t>
+          <t>0.47s</t>
         </is>
       </c>
       <c r="L3" s="17" t="inlineStr">
@@ -10796,7 +10866,7 @@
       </c>
       <c r="K4" s="7" t="inlineStr">
         <is>
-          <t>0.65s</t>
+          <t>1.17s</t>
         </is>
       </c>
       <c r="L4" s="15" t="inlineStr">
@@ -10866,7 +10936,7 @@
       </c>
       <c r="K5" s="11" t="inlineStr">
         <is>
-          <t>0.49s</t>
+          <t>1.22s</t>
         </is>
       </c>
       <c r="L5" s="17" t="inlineStr">
@@ -10936,7 +11006,7 @@
       </c>
       <c r="K6" s="7" t="inlineStr">
         <is>
-          <t>0.28s</t>
+          <t>1.10s</t>
         </is>
       </c>
       <c r="L6" s="15" t="inlineStr">
@@ -11006,7 +11076,7 @@
       </c>
       <c r="K7" s="11" t="inlineStr">
         <is>
-          <t>0.67s</t>
+          <t>0.90s</t>
         </is>
       </c>
       <c r="L7" s="17" t="inlineStr">
@@ -11076,7 +11146,7 @@
       </c>
       <c r="K8" s="7" t="inlineStr">
         <is>
-          <t>0.70s</t>
+          <t>0.20s</t>
         </is>
       </c>
       <c r="L8" s="15" t="inlineStr">
@@ -11146,7 +11216,7 @@
       </c>
       <c r="K9" s="11" t="inlineStr">
         <is>
-          <t>0.64s</t>
+          <t>0.67s</t>
         </is>
       </c>
       <c r="L9" s="17" t="inlineStr">
@@ -11216,7 +11286,7 @@
       </c>
       <c r="K10" s="7" t="inlineStr">
         <is>
-          <t>0.29s</t>
+          <t>1.19s</t>
         </is>
       </c>
       <c r="L10" s="15" t="inlineStr">
@@ -11286,7 +11356,7 @@
       </c>
       <c r="K11" s="11" t="inlineStr">
         <is>
-          <t>0.74s</t>
+          <t>0.29s</t>
         </is>
       </c>
       <c r="L11" s="17" t="inlineStr">
@@ -11356,7 +11426,7 @@
       </c>
       <c r="K12" s="7" t="inlineStr">
         <is>
-          <t>0.57s</t>
+          <t>0.64s</t>
         </is>
       </c>
       <c r="L12" s="15" t="inlineStr">
@@ -11426,7 +11496,7 @@
       </c>
       <c r="K13" s="11" t="inlineStr">
         <is>
-          <t>0.26s</t>
+          <t>0.21s</t>
         </is>
       </c>
       <c r="L13" s="17" t="inlineStr">
@@ -11496,7 +11566,7 @@
       </c>
       <c r="K14" s="7" t="inlineStr">
         <is>
-          <t>1.21s</t>
+          <t>0.52s</t>
         </is>
       </c>
       <c r="L14" s="15" t="inlineStr">
@@ -11566,7 +11636,7 @@
       </c>
       <c r="K15" s="11" t="inlineStr">
         <is>
-          <t>0.27s</t>
+          <t>0.60s</t>
         </is>
       </c>
       <c r="L15" s="17" t="inlineStr">
@@ -11636,7 +11706,7 @@
       </c>
       <c r="K16" s="7" t="inlineStr">
         <is>
-          <t>0.84s</t>
+          <t>0.58s</t>
         </is>
       </c>
       <c r="L16" s="15" t="inlineStr">
@@ -11802,7 +11872,7 @@
       </c>
       <c r="K2" s="7" t="inlineStr">
         <is>
-          <t>0.30s</t>
+          <t>0.47s</t>
         </is>
       </c>
       <c r="L2" s="15" t="inlineStr">
@@ -11872,7 +11942,7 @@
       </c>
       <c r="K3" s="11" t="inlineStr">
         <is>
-          <t>0.51s</t>
+          <t>0.92s</t>
         </is>
       </c>
       <c r="L3" s="17" t="inlineStr">
@@ -11942,7 +12012,7 @@
       </c>
       <c r="K4" s="7" t="inlineStr">
         <is>
-          <t>0.82s</t>
+          <t>0.18s</t>
         </is>
       </c>
       <c r="L4" s="15" t="inlineStr">
@@ -12012,7 +12082,7 @@
       </c>
       <c r="K5" s="11" t="inlineStr">
         <is>
-          <t>0.90s</t>
+          <t>0.26s</t>
         </is>
       </c>
       <c r="L5" s="17" t="inlineStr">
@@ -12082,7 +12152,7 @@
       </c>
       <c r="K6" s="7" t="inlineStr">
         <is>
-          <t>1.11s</t>
+          <t>0.59s</t>
         </is>
       </c>
       <c r="L6" s="15" t="inlineStr">
@@ -12152,7 +12222,7 @@
       </c>
       <c r="K7" s="11" t="inlineStr">
         <is>
-          <t>0.32s</t>
+          <t>1.07s</t>
         </is>
       </c>
       <c r="L7" s="17" t="inlineStr">
@@ -12222,7 +12292,7 @@
       </c>
       <c r="K8" s="7" t="inlineStr">
         <is>
-          <t>0.74s</t>
+          <t>0.45s</t>
         </is>
       </c>
       <c r="L8" s="15" t="inlineStr">
@@ -12292,7 +12362,7 @@
       </c>
       <c r="K9" s="11" t="inlineStr">
         <is>
-          <t>1.22s</t>
+          <t>0.66s</t>
         </is>
       </c>
       <c r="L9" s="17" t="inlineStr">
@@ -12362,7 +12432,7 @@
       </c>
       <c r="K10" s="7" t="inlineStr">
         <is>
-          <t>0.23s</t>
+          <t>0.58s</t>
         </is>
       </c>
       <c r="L10" s="15" t="inlineStr">
@@ -12432,7 +12502,7 @@
       </c>
       <c r="K11" s="11" t="inlineStr">
         <is>
-          <t>1.17s</t>
+          <t>0.81s</t>
         </is>
       </c>
       <c r="L11" s="17" t="inlineStr">
@@ -12502,7 +12572,7 @@
       </c>
       <c r="K12" s="7" t="inlineStr">
         <is>
-          <t>0.93s</t>
+          <t>0.95s</t>
         </is>
       </c>
       <c r="L12" s="15" t="inlineStr">
@@ -12572,7 +12642,7 @@
       </c>
       <c r="K13" s="11" t="inlineStr">
         <is>
-          <t>0.51s</t>
+          <t>1.17s</t>
         </is>
       </c>
       <c r="L13" s="17" t="inlineStr">
@@ -12642,7 +12712,7 @@
       </c>
       <c r="K14" s="7" t="inlineStr">
         <is>
-          <t>0.54s</t>
+          <t>0.60s</t>
         </is>
       </c>
       <c r="L14" s="15" t="inlineStr">
@@ -12712,7 +12782,7 @@
       </c>
       <c r="K15" s="11" t="inlineStr">
         <is>
-          <t>0.66s</t>
+          <t>0.60s</t>
         </is>
       </c>
       <c r="L15" s="17" t="inlineStr">
@@ -12782,7 +12852,7 @@
       </c>
       <c r="K16" s="7" t="inlineStr">
         <is>
-          <t>0.92s</t>
+          <t>0.14s</t>
         </is>
       </c>
       <c r="L16" s="15" t="inlineStr">
@@ -12807,7 +12877,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -12868,60 +12938,6 @@
       <c r="E2" s="15" t="inlineStr">
         <is>
           <t>LOGCAT_ERROR: Step 'Verify validation scenario 18 for Functional' failed during verification. Reason: API call timed out due to unstable backend sync.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="10" t="inlineStr">
-        <is>
-          <t>TC_FUNC_031</t>
-        </is>
-      </c>
-      <c r="B3" s="17" t="inlineStr">
-        <is>
-          <t>API call timed out due to unstable backend sync.</t>
-        </is>
-      </c>
-      <c r="C3" s="17" t="inlineStr">
-        <is>
-          <t>testing/appium/screenshots/tc_func_031.png</t>
-        </is>
-      </c>
-      <c r="D3" s="18" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="E3" s="17" t="inlineStr">
-        <is>
-          <t>LOGCAT_ERROR: Step 'Verify validation scenario 31 for Functional' failed during verification. Reason: API call timed out due to unstable backend sync.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>TC_UI_014</t>
-        </is>
-      </c>
-      <c r="B4" s="15" t="inlineStr">
-        <is>
-          <t>Text wrap overlaps on low-resolution views.</t>
-        </is>
-      </c>
-      <c r="C4" s="15" t="inlineStr">
-        <is>
-          <t>testing/appium/screenshots/tc_ui_014.png</t>
-        </is>
-      </c>
-      <c r="D4" s="18" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="E4" s="15" t="inlineStr">
-        <is>
-          <t>LOGCAT_ERROR: Step 'Verify validation scenario 14 for UI' failed during verification. Reason: Text wrap overlaps on low-resolution views.</t>
         </is>
       </c>
     </row>

</xml_diff>